<commit_message>
US_08 TC_12/13 sonuclari ve SCRUM-254 ile test case dosyasi guncellendi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Snack_Attack_Test_Cases_Yildiray_Kosedag.xlsx
+++ b/docs/Snack_Attack_Test_Cases_Yildiray_Kosedag.xlsx
@@ -34234,9 +34234,9 @@
         </is>
       </c>
       <c r="I1310" s="4" t="n"/>
-      <c r="J1310" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1310" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -34423,7 +34423,7 @@
       </c>
       <c r="I1318" s="4" t="inlineStr">
         <is>
-          <t>Bloke – sipariş oluşturulamadığı için (SCRUM-232) iptal senaryosu koşulamadı. (Bug: SCRUM-232)</t>
+          <t>UI'daki SCRUM-232 nedeniyle API ile oluşturulan Order #2'de Cancel Order'a basıldı, onay penceresi açıldı; Tamam sonrası "Order cancelled successfully." görüntülendi, durum CANCELED oldu (UI + API).</t>
         </is>
       </c>
       <c r="J1318" s="8" t="n"/>
@@ -34523,9 +34523,9 @@
         </is>
       </c>
       <c r="I1321" s="4" t="n"/>
-      <c r="J1321" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1321" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -34690,7 +34690,7 @@
       </c>
       <c r="I1328" s="4" t="inlineStr">
         <is>
-          <t>Bloke – sipariş oluşturulamadığı için (SCRUM-232) iptal senaryosu koşulamadı. (Bug: SCRUM-232)</t>
+          <t>CANCELED Order #2'de Cancel Order butonu görünür ve aktif kaldı; tekrar tıklanınca yalnızca "Failed to cancel the order." görüntülendi (durum değişmedi). (Bug: SCRUM-254)</t>
         </is>
       </c>
       <c r="J1328" s="8" t="n"/>
@@ -34957,7 +34957,7 @@
       </c>
       <c r="I1338" s="4" t="inlineStr">
         <is>
-          <t>Bloke – sipariş oluşturulamadığı için (SCRUM-232) iptal senaryosu koşulamadı. (Bug: SCRUM-232)</t>
+          <t>Bloke – CONFIRMED/DELIVERED durumunda sipariş için Admin/Seller hesabı gerekli.</t>
         </is>
       </c>
       <c r="J1338" s="8" t="n"/>
@@ -35224,7 +35224,7 @@
       </c>
       <c r="I1348" s="4" t="inlineStr">
         <is>
-          <t>Bloke – sipariş oluşturulamadığı için (SCRUM-232) iptal senaryosu koşulamadı. (Bug: SCRUM-232)</t>
+          <t>Bloke – CONFIRMED/DELIVERED durumunda sipariş için Admin/Seller hesabı gerekli.</t>
         </is>
       </c>
       <c r="J1348" s="8" t="n"/>
@@ -67169,13 +67169,13 @@
         <v>5</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K9" s="4" t="n">
         <v>0</v>
@@ -67759,13 +67759,13 @@
         <v>91</v>
       </c>
       <c r="H23" s="12" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J23" s="12" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K23" s="12" t="n">
         <v>114</v>

</xml_diff>

<commit_message>
US_05 profil testleri ve SCRUM-255/256 ile test case dosyasi guncellendi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Snack_Attack_Test_Cases_Yildiray_Kosedag.xlsx
+++ b/docs/Snack_Attack_Test_Cases_Yildiray_Kosedag.xlsx
@@ -23013,7 +23013,11 @@
         </is>
       </c>
       <c r="I885" s="4" t="n"/>
-      <c r="J885" s="2" t="n"/>
+      <c r="J885" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
     </row>
     <row r="886">
       <c r="A886" s="7" t="n"/>
@@ -23244,7 +23248,11 @@
           <t>Username alanında güncel data görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I895" s="4" t="n"/>
+      <c r="I895" s="4" t="inlineStr">
+        <is>
+          <t>Username "yildiray54qa" yapıldı, şifre girilip Update Profile tıklandı: "User is updated Successfully" görüntülendi; sayfa yenilenince ve API'de yeni username görüntülendi (sonra eski değere döndürüldü). Not: güncelleme için şifre girilmesi zorunlu.</t>
+        </is>
+      </c>
       <c r="J895" s="8" t="n"/>
     </row>
     <row r="897">
@@ -23341,7 +23349,11 @@
         </is>
       </c>
       <c r="I898" s="4" t="n"/>
-      <c r="J898" s="2" t="n"/>
+      <c r="J898" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
     </row>
     <row r="899">
       <c r="A899" s="7" t="n"/>
@@ -23572,7 +23584,11 @@
           <t>Email alanında güncel data görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I908" s="4" t="n"/>
+      <c r="I908" s="4" t="inlineStr">
+        <is>
+          <t>Email alanı klavye girişini kabul etmiyor; yazılan değer anında eski email'e dönüyor, güncelleme yapılamadı. (Bug: SCRUM-256)</t>
+        </is>
+      </c>
       <c r="J908" s="8" t="n"/>
     </row>
     <row r="910">
@@ -23669,7 +23685,11 @@
         </is>
       </c>
       <c r="I911" s="4" t="n"/>
-      <c r="J911" s="2" t="n"/>
+      <c r="J911" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
     </row>
     <row r="912">
       <c r="A912" s="7" t="n"/>
@@ -23900,7 +23920,11 @@
           <t>First Name alanında güncel data görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I921" s="4" t="n"/>
+      <c r="I921" s="4" t="inlineStr">
+        <is>
+          <t>First Name değiştirildi, "User is updated Successfully" görüntülendi ancak sayfa yenilenince ve API'de eski değer görüntülendi; First Name kaydedilmiyor (2 kez tekrarlandı). (Bug: SCRUM-255)</t>
+        </is>
+      </c>
       <c r="J921" s="8" t="n"/>
     </row>
     <row r="923">
@@ -23997,7 +24021,11 @@
         </is>
       </c>
       <c r="I924" s="4" t="n"/>
-      <c r="J924" s="2" t="n"/>
+      <c r="J924" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
     </row>
     <row r="925">
       <c r="A925" s="7" t="n"/>
@@ -24228,7 +24256,11 @@
           <t>Last Name alanında güncel data görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I934" s="4" t="n"/>
+      <c r="I934" s="4" t="inlineStr">
+        <is>
+          <t>Last Name değiştirildi, "User is updated Successfully" görüntülendi ancak sayfa yenilenince ve API'de eski değer görüntülendi; Last Name kaydedilmiyor (2 kez tekrarlandı). (Bug: SCRUM-255)</t>
+        </is>
+      </c>
       <c r="J934" s="8" t="n"/>
     </row>
     <row r="936">
@@ -24325,7 +24357,11 @@
         </is>
       </c>
       <c r="I937" s="4" t="n"/>
-      <c r="J937" s="2" t="n"/>
+      <c r="J937" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
     </row>
     <row r="938">
       <c r="A938" s="7" t="n"/>
@@ -24556,7 +24592,11 @@
           <t>Address alanında güncel data görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I947" s="4" t="n"/>
+      <c r="I947" s="4" t="inlineStr">
+        <is>
+          <t>Address değiştirildi, "User is updated Successfully" görüntülendi ancak sayfa yenilenince ve API'de eski değer görüntülendi; Address kaydedilmiyor (2 kez tekrarlandı). (Bug: SCRUM-255)</t>
+        </is>
+      </c>
       <c r="J947" s="8" t="n"/>
     </row>
     <row r="949">
@@ -24653,7 +24693,11 @@
         </is>
       </c>
       <c r="I950" s="4" t="n"/>
-      <c r="J950" s="2" t="n"/>
+      <c r="J950" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
     </row>
     <row r="951">
       <c r="A951" s="7" t="n"/>
@@ -24884,7 +24928,11 @@
           <t>Phone Number alanında güncel data görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I960" s="4" t="n"/>
+      <c r="I960" s="4" t="inlineStr">
+        <is>
+          <t>Phone Number "5418921175" yapıldı, "User is updated Successfully" görüntülendi; yenilemede ve API'de yeni numara görüntülendi (sonra eski değere döndürüldü).</t>
+        </is>
+      </c>
       <c r="J960" s="8" t="n"/>
     </row>
     <row r="962">
@@ -24981,7 +25029,11 @@
         </is>
       </c>
       <c r="I963" s="4" t="n"/>
-      <c r="J963" s="2" t="n"/>
+      <c r="J963" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
     </row>
     <row r="964">
       <c r="A964" s="7" t="n"/>
@@ -25238,7 +25290,11 @@
           <t>Kullanıcı yeni şifre ile giriş yapabilmelidir</t>
         </is>
       </c>
-      <c r="I974" s="4" t="n"/>
+      <c r="I974" s="4" t="inlineStr">
+        <is>
+          <t>Password alanına yeni şifre girilip Update Profile tıklandı, "User is updated Successfully" görüntülendi; çıkış yapılıp yeni şifre ile giriş yapıldığında "Login successful!" görüntülendi.</t>
+        </is>
+      </c>
       <c r="J974" s="8" t="n"/>
     </row>
     <row r="976">
@@ -25335,7 +25391,11 @@
         </is>
       </c>
       <c r="I977" s="4" t="n"/>
-      <c r="J977" s="2" t="n"/>
+      <c r="J977" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
     </row>
     <row r="978">
       <c r="A978" s="7" t="n"/>
@@ -25544,7 +25604,11 @@
           <t>"User is updated successfully" mesajı görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I986" s="4" t="n"/>
+      <c r="I986" s="4" t="inlineStr">
+        <is>
+          <t>Username, First Name, Last Name, Address ve Phone aynı anda değiştirildi; başarı mesajı görüntülendi ancak yalnızca Username ve Phone kaydedildi, First/Last Name ve Address eski değerinde kaldı; updatedAt güncellenmedi. (Bug: SCRUM-255)</t>
+        </is>
+      </c>
       <c r="J986" s="8" t="n"/>
     </row>
     <row r="988">
@@ -25856,7 +25920,7 @@
       </c>
       <c r="I998" s="4" t="inlineStr">
         <is>
-          <t>Email alanına "yildiraymail" girildiğinde tarayıcı doğrulaması ("@ işareti eksik") güncellemeyi engelledi.</t>
+          <t>Email alanına "yildiraymail" girildiğinde tarayıcı doğrulaması ("@ işareti eksik") güncellemeyi engelledi. Not: Email alanı klavyeyle düzenlenemiyor (SCRUM-256).</t>
         </is>
       </c>
       <c r="J998" s="8" t="n"/>
@@ -67040,16 +67104,16 @@
         <v>2</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -67759,16 +67823,16 @@
         <v>91</v>
       </c>
       <c r="H23" s="12" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="J23" s="12" t="n">
         <v>4</v>
       </c>
       <c r="K23" s="12" t="n">
-        <v>114</v>
+        <v>106</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
Test Plani'na Test Ozet Raporu eklendi; admin testleri BLOCKED olarak isaretlendi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Snack_Attack_Test_Cases_Yildiray_Kosedag.xlsx
+++ b/docs/Snack_Attack_Test_Cases_Yildiray_Kosedag.xlsx
@@ -10915,7 +10915,11 @@
         </is>
       </c>
       <c r="I400" s="4" t="n"/>
-      <c r="J400" s="2" t="n"/>
+      <c r="J400" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="401">
       <c r="A401" s="7" t="n"/>
@@ -11354,7 +11358,11 @@
           <t>"Success" mesajı görüntülenmeli ve kayıt işlemi başarılı olmalıdır</t>
         </is>
       </c>
-      <c r="I418" s="4" t="n"/>
+      <c r="I418" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J418" s="8" t="n"/>
     </row>
     <row r="419">
@@ -11459,7 +11467,11 @@
         </is>
       </c>
       <c r="I422" s="4" t="n"/>
-      <c r="J422" s="2" t="n"/>
+      <c r="J422" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="423">
       <c r="A423" s="7" t="n"/>
@@ -11894,7 +11906,11 @@
           <t>Kayıt işlemi başarısız olmalı, kullanıcı kayıt sayfasında kalmalıdır</t>
         </is>
       </c>
-      <c r="I440" s="4" t="n"/>
+      <c r="I440" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J440" s="8" t="n"/>
     </row>
     <row r="441">
@@ -11999,7 +12015,11 @@
         </is>
       </c>
       <c r="I444" s="4" t="n"/>
-      <c r="J444" s="2" t="n"/>
+      <c r="J444" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="445">
       <c r="A445" s="7" t="n"/>
@@ -12434,7 +12454,11 @@
           <t>Kayıt işlemi başarısız olmalı, kullanıcı kayıt sayfasında kalmalıdır</t>
         </is>
       </c>
-      <c r="I462" s="4" t="n"/>
+      <c r="I462" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J462" s="8" t="n"/>
     </row>
     <row r="463">
@@ -12539,7 +12563,11 @@
         </is>
       </c>
       <c r="I466" s="4" t="n"/>
-      <c r="J466" s="2" t="n"/>
+      <c r="J466" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="467">
       <c r="A467" s="7" t="n"/>
@@ -12974,7 +13002,11 @@
           <t>Kayıt işlemi başarısız olmalı, kullanıcı kayıt sayfasında kalmalıdır</t>
         </is>
       </c>
-      <c r="I484" s="4" t="n"/>
+      <c r="I484" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J484" s="8" t="n"/>
     </row>
     <row r="485">
@@ -13079,7 +13111,11 @@
         </is>
       </c>
       <c r="I488" s="4" t="n"/>
-      <c r="J488" s="2" t="n"/>
+      <c r="J488" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="489">
       <c r="A489" s="7" t="n"/>
@@ -13514,7 +13550,11 @@
           <t>Kayıt işlemi başarısız olmalı, kullanıcı kayıt sayfasında kalmalıdır</t>
         </is>
       </c>
-      <c r="I506" s="4" t="n"/>
+      <c r="I506" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J506" s="8" t="n"/>
     </row>
     <row r="507">
@@ -13619,7 +13659,11 @@
         </is>
       </c>
       <c r="I510" s="4" t="n"/>
-      <c r="J510" s="2" t="n"/>
+      <c r="J510" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="511">
       <c r="A511" s="7" t="n"/>
@@ -14054,7 +14098,11 @@
           <t>Kayıt işlemi başarısız olmalı, kullanıcı kayıt sayfasında kalmalıdır</t>
         </is>
       </c>
-      <c r="I528" s="4" t="n"/>
+      <c r="I528" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J528" s="8" t="n"/>
     </row>
     <row r="529">
@@ -14159,7 +14207,11 @@
         </is>
       </c>
       <c r="I532" s="4" t="n"/>
-      <c r="J532" s="2" t="n"/>
+      <c r="J532" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="533">
       <c r="A533" s="7" t="n"/>
@@ -14594,7 +14646,11 @@
           <t>Kayıt işlemi başarısız olmalı, kullanıcı kayıt sayfasında kalmalıdır</t>
         </is>
       </c>
-      <c r="I550" s="4" t="n"/>
+      <c r="I550" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J550" s="8" t="n"/>
     </row>
     <row r="551">
@@ -14699,7 +14755,11 @@
         </is>
       </c>
       <c r="I554" s="4" t="n"/>
-      <c r="J554" s="2" t="n"/>
+      <c r="J554" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="555">
       <c r="A555" s="7" t="n"/>
@@ -15134,7 +15194,11 @@
           <t>Kayıt işlemi başarısız olmalı, kullanıcı kayıt sayfasında kalmalıdır</t>
         </is>
       </c>
-      <c r="I572" s="4" t="n"/>
+      <c r="I572" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J572" s="8" t="n"/>
     </row>
     <row r="573">
@@ -15239,7 +15303,11 @@
         </is>
       </c>
       <c r="I576" s="4" t="n"/>
-      <c r="J576" s="2" t="n"/>
+      <c r="J576" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="577">
       <c r="A577" s="7" t="n"/>
@@ -15678,7 +15746,11 @@
           <t>Kayıt işlemi başarısız olmalı, kullanıcı kayıt sayfasında kalmalıdır</t>
         </is>
       </c>
-      <c r="I594" s="4" t="n"/>
+      <c r="I594" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J594" s="8" t="n"/>
     </row>
     <row r="595">
@@ -15783,7 +15855,11 @@
         </is>
       </c>
       <c r="I598" s="4" t="n"/>
-      <c r="J598" s="2" t="n"/>
+      <c r="J598" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="599">
       <c r="A599" s="7" t="n"/>
@@ -16222,7 +16298,11 @@
           <t>Kayıt işlemi başarısız olmalı, kullanıcı kayıt sayfasında kalmalıdır</t>
         </is>
       </c>
-      <c r="I616" s="4" t="n"/>
+      <c r="I616" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J616" s="8" t="n"/>
     </row>
     <row r="617">
@@ -16327,7 +16407,11 @@
         </is>
       </c>
       <c r="I620" s="4" t="n"/>
-      <c r="J620" s="2" t="n"/>
+      <c r="J620" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="621">
       <c r="A621" s="7" t="n"/>
@@ -16766,7 +16850,11 @@
           <t>Kayıt işlemi başarısız olmalı, kullanıcı kayıt sayfasında kalmalıdır</t>
         </is>
       </c>
-      <c r="I638" s="4" t="n"/>
+      <c r="I638" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J638" s="8" t="n"/>
     </row>
     <row r="639">
@@ -16871,7 +16959,11 @@
         </is>
       </c>
       <c r="I642" s="4" t="n"/>
-      <c r="J642" s="2" t="n"/>
+      <c r="J642" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="643">
       <c r="A643" s="7" t="n"/>
@@ -17310,7 +17402,11 @@
           <t>Kayıt işlemi başarısız olmalı, kullanıcı kayıt sayfasında kalmalıdır</t>
         </is>
       </c>
-      <c r="I660" s="4" t="n"/>
+      <c r="I660" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J660" s="8" t="n"/>
     </row>
     <row r="661">
@@ -17415,7 +17511,11 @@
         </is>
       </c>
       <c r="I664" s="4" t="n"/>
-      <c r="J664" s="2" t="n"/>
+      <c r="J664" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="665">
       <c r="A665" s="7" t="n"/>
@@ -17854,7 +17954,11 @@
           <t>Kayıt işlemi başarısız olmalı, kullanıcı kayıt sayfasında kalmalıdır</t>
         </is>
       </c>
-      <c r="I682" s="4" t="n"/>
+      <c r="I682" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J682" s="8" t="n"/>
     </row>
     <row r="683">
@@ -17959,7 +18063,11 @@
         </is>
       </c>
       <c r="I686" s="4" t="n"/>
-      <c r="J686" s="2" t="n"/>
+      <c r="J686" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="687">
       <c r="A687" s="7" t="n"/>
@@ -18398,7 +18506,11 @@
           <t>Kayıt işlemi başarısız olmalı, kullanıcı kayıt sayfasında kalmalıdır</t>
         </is>
       </c>
-      <c r="I704" s="4" t="n"/>
+      <c r="I704" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J704" s="8" t="n"/>
     </row>
     <row r="705">
@@ -18503,7 +18615,11 @@
         </is>
       </c>
       <c r="I708" s="4" t="n"/>
-      <c r="J708" s="2" t="n"/>
+      <c r="J708" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="709">
       <c r="A709" s="7" t="n"/>
@@ -18938,7 +19054,11 @@
           <t>Kayıt işlemi başarısız olmalı, kullanıcı kayıt sayfasında kalmalıdır</t>
         </is>
       </c>
-      <c r="I726" s="4" t="n"/>
+      <c r="I726" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J726" s="8" t="n"/>
     </row>
     <row r="727">
@@ -19043,7 +19163,11 @@
         </is>
       </c>
       <c r="I730" s="4" t="n"/>
-      <c r="J730" s="2" t="n"/>
+      <c r="J730" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="731">
       <c r="A731" s="7" t="n"/>
@@ -19478,7 +19602,11 @@
           <t>Kayıt işlemi başarısız olmalı, kullanıcı kayıt sayfasında kalmalıdır</t>
         </is>
       </c>
-      <c r="I748" s="4" t="n"/>
+      <c r="I748" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J748" s="8" t="n"/>
     </row>
     <row r="749">
@@ -19583,7 +19711,11 @@
         </is>
       </c>
       <c r="I752" s="4" t="n"/>
-      <c r="J752" s="2" t="n"/>
+      <c r="J752" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="753">
       <c r="A753" s="7" t="n"/>
@@ -20022,7 +20154,11 @@
           <t>Kayıt işlemi başarısız olmalı, kullanıcı kayıt sayfasında kalmalıdır</t>
         </is>
       </c>
-      <c r="I770" s="4" t="n"/>
+      <c r="I770" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J770" s="8" t="n"/>
     </row>
     <row r="771">
@@ -20126,7 +20262,11 @@
         </is>
       </c>
       <c r="I774" s="4" t="n"/>
-      <c r="J774" s="2" t="n"/>
+      <c r="J774" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="775">
       <c r="A775" s="7" t="n"/>
@@ -20565,7 +20705,11 @@
           <t>Email'in zaten kayıtlı olduğuna dair uyarı mesajı görüntülenmeli, kayıt yapılmamalıdır</t>
         </is>
       </c>
-      <c r="I792" s="4" t="n"/>
+      <c r="I792" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J792" s="8" t="n"/>
     </row>
     <row r="793">
@@ -20670,7 +20814,11 @@
         </is>
       </c>
       <c r="I796" s="4" t="n"/>
-      <c r="J796" s="2" t="n"/>
+      <c r="J796" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="797">
       <c r="A797" s="7" t="n"/>
@@ -20883,7 +21031,11 @@
           <t>Girilen şifre maskelenmiş (●●●) olarak görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I805" s="4" t="n"/>
+      <c r="I805" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J805" s="8" t="n"/>
     </row>
     <row r="807">
@@ -20980,7 +21132,11 @@
         </is>
       </c>
       <c r="I808" s="4" t="n"/>
-      <c r="J808" s="2" t="n"/>
+      <c r="J808" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="809">
       <c r="A809" s="7" t="n"/>
@@ -21119,7 +21275,11 @@
           <t>Admin Dashboard sayfası görüntülenebilmelidir</t>
         </is>
       </c>
-      <c r="I814" s="4" t="n"/>
+      <c r="I814" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J814" s="8" t="n"/>
     </row>
     <row r="815">
@@ -21223,7 +21383,11 @@
         </is>
       </c>
       <c r="I818" s="4" t="n"/>
-      <c r="J818" s="2" t="n"/>
+      <c r="J818" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="819">
       <c r="A819" s="7" t="n"/>
@@ -21340,7 +21504,11 @@
           <t>Email alanının altında "Invalid email" uyarı metni görüntülenmeli, giriş yapılmamalıdır</t>
         </is>
       </c>
-      <c r="I823" s="4" t="n"/>
+      <c r="I823" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J823" s="8" t="n"/>
     </row>
     <row r="825">
@@ -21437,7 +21605,11 @@
         </is>
       </c>
       <c r="I826" s="4" t="n"/>
-      <c r="J826" s="2" t="n"/>
+      <c r="J826" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="827">
       <c r="A827" s="7" t="n"/>
@@ -21554,7 +21726,11 @@
           <t>Email alanının altında "Invalid email" uyarı metni görüntülenmeli, giriş yapılmamalıdır</t>
         </is>
       </c>
-      <c r="I831" s="4" t="n"/>
+      <c r="I831" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J831" s="8" t="n"/>
     </row>
     <row r="833">
@@ -21651,7 +21827,11 @@
         </is>
       </c>
       <c r="I834" s="4" t="n"/>
-      <c r="J834" s="2" t="n"/>
+      <c r="J834" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="835">
       <c r="A835" s="7" t="n"/>
@@ -21764,7 +21944,11 @@
           <t>Password alanının altında "Password is required" uyarı metni görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I839" s="4" t="n"/>
+      <c r="I839" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J839" s="8" t="n"/>
     </row>
     <row r="841">
@@ -21861,7 +22045,11 @@
         </is>
       </c>
       <c r="I842" s="4" t="n"/>
-      <c r="J842" s="2" t="n"/>
+      <c r="J842" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="843">
       <c r="A843" s="7" t="n"/>
@@ -21948,7 +22136,11 @@
           <t>Login butonu pasif (disabled) olmalı, tıklanamamalıdır</t>
         </is>
       </c>
-      <c r="I846" s="4" t="n"/>
+      <c r="I846" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J846" s="8" t="n"/>
     </row>
     <row r="848">
@@ -22045,7 +22237,11 @@
         </is>
       </c>
       <c r="I849" s="4" t="n"/>
-      <c r="J849" s="2" t="n"/>
+      <c r="J849" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="850">
       <c r="A850" s="7" t="n"/>
@@ -22136,7 +22332,11 @@
           <t>Login butonu pasif (disabled) olmalıdır</t>
         </is>
       </c>
-      <c r="I853" s="4" t="n"/>
+      <c r="I853" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J853" s="8" t="n"/>
     </row>
     <row r="855">
@@ -22233,7 +22433,11 @@
         </is>
       </c>
       <c r="I856" s="4" t="n"/>
-      <c r="J856" s="2" t="n"/>
+      <c r="J856" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="857">
       <c r="A857" s="7" t="n"/>
@@ -22324,7 +22528,11 @@
           <t>Login butonu pasif (disabled) olmalıdır</t>
         </is>
       </c>
-      <c r="I860" s="4" t="n"/>
+      <c r="I860" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J860" s="8" t="n"/>
     </row>
     <row r="862">
@@ -22421,7 +22629,11 @@
         </is>
       </c>
       <c r="I863" s="4" t="n"/>
-      <c r="J863" s="2" t="n"/>
+      <c r="J863" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="864">
       <c r="A864" s="7" t="n"/>
@@ -22538,7 +22750,11 @@
           <t>Giriş yapılmamalı; login sayfasında anlaşılır bir hata mesajı (ör. "Sign in failed. Check the details you provided are correct.") görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I868" s="4" t="n"/>
+      <c r="I868" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J868" s="8" t="n"/>
     </row>
     <row r="870">
@@ -22634,7 +22850,11 @@
         </is>
       </c>
       <c r="I871" s="4" t="n"/>
-      <c r="J871" s="2" t="n"/>
+      <c r="J871" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="872">
       <c r="A872" s="7" t="n"/>
@@ -22751,7 +22971,11 @@
           <t>Giriş yapılmamalı; login sayfasında anlaşılır bir hata mesajı görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I876" s="4" t="n"/>
+      <c r="I876" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J876" s="8" t="n"/>
     </row>
     <row r="878">
@@ -22847,7 +23071,11 @@
         </is>
       </c>
       <c r="I879" s="4" t="n"/>
-      <c r="J879" s="2" t="n"/>
+      <c r="J879" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="880">
       <c r="A880" s="7" t="n"/>
@@ -22916,7 +23144,11 @@
           <t>Şifre maskelenmiş (●●●) olarak görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I882" s="4" t="n"/>
+      <c r="I882" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J882" s="8" t="n"/>
     </row>
     <row r="884">
@@ -37122,7 +37354,11 @@
         </is>
       </c>
       <c r="I1417" s="4" t="n"/>
-      <c r="J1417" s="2" t="n"/>
+      <c r="J1417" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1418">
       <c r="A1418" s="7" t="n"/>
@@ -37331,7 +37567,11 @@
           <t>User ID, Email, First Name, Last Name, Phone Number kolonları ve dataları görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1426" s="4" t="n"/>
+      <c r="I1426" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1426" s="8" t="n"/>
     </row>
     <row r="1428">
@@ -37428,7 +37668,11 @@
         </is>
       </c>
       <c r="I1429" s="4" t="n"/>
-      <c r="J1429" s="2" t="n"/>
+      <c r="J1429" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1430">
       <c r="A1430" s="7" t="n"/>
@@ -37637,7 +37881,11 @@
           <t>Diğer kayıtlar listelenmelidir</t>
         </is>
       </c>
-      <c r="I1438" s="4" t="n"/>
+      <c r="I1438" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1438" s="8" t="n"/>
     </row>
     <row r="1440">
@@ -37735,7 +37983,11 @@
         </is>
       </c>
       <c r="I1441" s="4" t="n"/>
-      <c r="J1441" s="2" t="n"/>
+      <c r="J1441" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1442">
       <c r="A1442" s="7" t="n"/>
@@ -37966,7 +38218,11 @@
           <t>Başarı mesajı görüntülenmeli, hesap listeden kaldırılmalıdır</t>
         </is>
       </c>
-      <c r="I1451" s="4" t="n"/>
+      <c r="I1451" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1451" s="8" t="n"/>
     </row>
     <row r="1453">
@@ -38063,7 +38319,11 @@
         </is>
       </c>
       <c r="I1454" s="4" t="n"/>
-      <c r="J1454" s="2" t="n"/>
+      <c r="J1454" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1455">
       <c r="A1455" s="7" t="n"/>
@@ -38272,7 +38532,11 @@
           <t>Hesap silinmemeli, listede görüntülenmeye devam etmelidir</t>
         </is>
       </c>
-      <c r="I1463" s="4" t="n"/>
+      <c r="I1463" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1463" s="8" t="n"/>
     </row>
     <row r="1465">
@@ -38370,7 +38634,11 @@
         </is>
       </c>
       <c r="I1466" s="4" t="n"/>
-      <c r="J1466" s="2" t="n"/>
+      <c r="J1466" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1467">
       <c r="A1467" s="7" t="n"/>
@@ -38439,7 +38707,11 @@
           <t>Giriş yapılamamalıdır</t>
         </is>
       </c>
-      <c r="I1469" s="4" t="n"/>
+      <c r="I1469" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1469" s="8" t="n"/>
     </row>
     <row r="1471">
@@ -38536,7 +38808,11 @@
         </is>
       </c>
       <c r="I1472" s="4" t="n"/>
-      <c r="J1472" s="2" t="n"/>
+      <c r="J1472" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1473">
       <c r="A1473" s="7" t="n"/>
@@ -38745,7 +39021,11 @@
           <t>User ID, Email, First Name, Last Name, Phone Number kolonları ve dataları görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1481" s="4" t="n"/>
+      <c r="I1481" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1481" s="8" t="n"/>
     </row>
     <row r="1483">
@@ -38842,7 +39122,11 @@
         </is>
       </c>
       <c r="I1484" s="4" t="n"/>
-      <c r="J1484" s="2" t="n"/>
+      <c r="J1484" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1485">
       <c r="A1485" s="7" t="n"/>
@@ -39051,7 +39335,11 @@
           <t>Diğer kayıtlar listelenmelidir</t>
         </is>
       </c>
-      <c r="I1493" s="4" t="n"/>
+      <c r="I1493" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1493" s="8" t="n"/>
     </row>
     <row r="1495">
@@ -39149,7 +39437,11 @@
         </is>
       </c>
       <c r="I1496" s="4" t="n"/>
-      <c r="J1496" s="2" t="n"/>
+      <c r="J1496" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1497">
       <c r="A1497" s="7" t="n"/>
@@ -39380,7 +39672,11 @@
           <t>Başarı mesajı görüntülenmeli, hesap listeden kaldırılmalıdır</t>
         </is>
       </c>
-      <c r="I1506" s="4" t="n"/>
+      <c r="I1506" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1506" s="8" t="n"/>
     </row>
     <row r="1508">
@@ -39477,7 +39773,11 @@
         </is>
       </c>
       <c r="I1509" s="4" t="n"/>
-      <c r="J1509" s="2" t="n"/>
+      <c r="J1509" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1510">
       <c r="A1510" s="7" t="n"/>
@@ -39686,7 +39986,11 @@
           <t>Hesap silinmemeli, listede görüntülenmeye devam etmelidir</t>
         </is>
       </c>
-      <c r="I1518" s="4" t="n"/>
+      <c r="I1518" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1518" s="8" t="n"/>
     </row>
     <row r="1520">
@@ -39783,7 +40087,11 @@
         </is>
       </c>
       <c r="I1521" s="4" t="n"/>
-      <c r="J1521" s="2" t="n"/>
+      <c r="J1521" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1522">
       <c r="A1522" s="7" t="n"/>
@@ -39992,7 +40300,11 @@
           <t>Delete butonu pasif olmalı VEYA silinemeyeceğine dair uyarı görüntülenmeli; hesap silinmemelidir</t>
         </is>
       </c>
-      <c r="I1530" s="4" t="n"/>
+      <c r="I1530" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1530" s="8" t="n"/>
     </row>
     <row r="1532">
@@ -40089,7 +40401,11 @@
         </is>
       </c>
       <c r="I1533" s="4" t="n"/>
-      <c r="J1533" s="2" t="n"/>
+      <c r="J1533" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1534">
       <c r="A1534" s="7" t="n"/>
@@ -40272,7 +40588,11 @@
           <t>Payment, Total Price, Status ve Date bilgileri görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1541" s="4" t="n"/>
+      <c r="I1541" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1541" s="8" t="n"/>
     </row>
     <row r="1543">
@@ -40369,7 +40689,11 @@
         </is>
       </c>
       <c r="I1544" s="4" t="n"/>
-      <c r="J1544" s="2" t="n"/>
+      <c r="J1544" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1545">
       <c r="A1545" s="7" t="n"/>
@@ -40574,7 +40898,11 @@
           <t>Diğer siparişler listelenmelidir</t>
         </is>
       </c>
-      <c r="I1553" s="4" t="n"/>
+      <c r="I1553" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1553" s="8" t="n"/>
     </row>
     <row r="1555">
@@ -40671,7 +40999,11 @@
         </is>
       </c>
       <c r="I1556" s="4" t="n"/>
-      <c r="J1556" s="2" t="n"/>
+      <c r="J1556" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1557">
       <c r="A1557" s="7" t="n"/>
@@ -40876,7 +41208,11 @@
           <t>Sipariş kodu, kullanıcı, ürünler, ilaveler, adres, ödeme yöntemi, tutar ve statü görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1565" s="4" t="n"/>
+      <c r="I1565" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1565" s="8" t="n"/>
     </row>
     <row r="1567">
@@ -40974,7 +41310,11 @@
         </is>
       </c>
       <c r="I1568" s="4" t="n"/>
-      <c r="J1568" s="2" t="n"/>
+      <c r="J1568" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1569">
       <c r="A1569" s="7" t="n"/>
@@ -41205,7 +41545,11 @@
           <t>Kullanıcı tarafında da statü CONFIRMED görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1578" s="4" t="n"/>
+      <c r="I1578" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1578" s="8" t="n"/>
     </row>
     <row r="1580">
@@ -41303,7 +41647,11 @@
         </is>
       </c>
       <c r="I1581" s="4" t="n"/>
-      <c r="J1581" s="2" t="n"/>
+      <c r="J1581" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1582">
       <c r="A1582" s="7" t="n"/>
@@ -41534,7 +41882,11 @@
           <t>Kullanıcı tarafında da statü DELIVERED görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1591" s="4" t="n"/>
+      <c r="I1591" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1591" s="8" t="n"/>
     </row>
     <row r="1593">
@@ -41632,7 +41984,11 @@
         </is>
       </c>
       <c r="I1594" s="4" t="n"/>
-      <c r="J1594" s="2" t="n"/>
+      <c r="J1594" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1595">
       <c r="A1595" s="7" t="n"/>
@@ -41841,7 +42197,11 @@
           <t>Statü değiştirme seçeneği pasif olmalı VEYA uyarı görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1603" s="4" t="n"/>
+      <c r="I1603" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1603" s="8" t="n"/>
     </row>
     <row r="1605">
@@ -41938,7 +42298,11 @@
         </is>
       </c>
       <c r="I1606" s="4" t="n"/>
-      <c r="J1606" s="2" t="n"/>
+      <c r="J1606" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1607">
       <c r="A1607" s="7" t="n"/>
@@ -42121,7 +42485,11 @@
           <t>Ürün adı, kategori, fiyat, indirim, available/active durumu görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1614" s="4" t="n"/>
+      <c r="I1614" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1614" s="8" t="n"/>
     </row>
     <row r="1616">
@@ -42218,7 +42586,11 @@
         </is>
       </c>
       <c r="I1617" s="4" t="n"/>
-      <c r="J1617" s="2" t="n"/>
+      <c r="J1617" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1618">
       <c r="A1618" s="7" t="n"/>
@@ -42427,7 +42799,11 @@
           <t>Yalnızca seçilen kategorideki ürünler listelenmelidir</t>
         </is>
       </c>
-      <c r="I1626" s="4" t="n"/>
+      <c r="I1626" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1626" s="8" t="n"/>
     </row>
     <row r="1628">
@@ -42524,7 +42900,11 @@
         </is>
       </c>
       <c r="I1629" s="4" t="n"/>
-      <c r="J1629" s="2" t="n"/>
+      <c r="J1629" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1630">
       <c r="A1630" s="7" t="n"/>
@@ -42733,7 +43113,11 @@
           <t>Aranan ürün listelenmelidir</t>
         </is>
       </c>
-      <c r="I1638" s="4" t="n"/>
+      <c r="I1638" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1638" s="8" t="n"/>
     </row>
     <row r="1640">
@@ -42830,7 +43214,11 @@
         </is>
       </c>
       <c r="I1641" s="4" t="n"/>
-      <c r="J1641" s="2" t="n"/>
+      <c r="J1641" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1642">
       <c r="A1642" s="7" t="n"/>
@@ -43039,7 +43427,11 @@
           <t>Ürün listelenmemeli, bilgilendirme mesajı görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1650" s="4" t="n"/>
+      <c r="I1650" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1650" s="8" t="n"/>
     </row>
     <row r="1652">
@@ -43136,7 +43528,11 @@
         </is>
       </c>
       <c r="I1653" s="4" t="n"/>
-      <c r="J1653" s="2" t="n"/>
+      <c r="J1653" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1654">
       <c r="A1654" s="7" t="n"/>
@@ -43593,7 +43989,11 @@
           <t>Başarı mesajı görüntülenmeli, ürün listede ve kullanıcı Products sayfasında görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1672" s="4" t="n"/>
+      <c r="I1672" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1672" s="8" t="n"/>
     </row>
     <row r="1673">
@@ -43697,7 +44097,11 @@
         </is>
       </c>
       <c r="I1676" s="4" t="n"/>
-      <c r="J1676" s="2" t="n"/>
+      <c r="J1676" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1677">
       <c r="A1677" s="7" t="n"/>
@@ -44150,7 +44554,11 @@
           <t>Başarı mesajı görüntülenmeli, ürün listede ve kullanıcı Products sayfasında görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1695" s="4" t="n"/>
+      <c r="I1695" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1695" s="8" t="n"/>
     </row>
     <row r="1697">
@@ -44247,7 +44655,11 @@
         </is>
       </c>
       <c r="I1698" s="4" t="n"/>
-      <c r="J1698" s="2" t="n"/>
+      <c r="J1698" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1699">
       <c r="A1699" s="7" t="n"/>
@@ -44700,7 +45112,11 @@
           <t>Uyarı mesajı görüntülenmeli, ürün kaydedilmemelidir</t>
         </is>
       </c>
-      <c r="I1717" s="4" t="n"/>
+      <c r="I1717" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1717" s="8" t="n"/>
     </row>
     <row r="1719">
@@ -44797,7 +45213,11 @@
         </is>
       </c>
       <c r="I1720" s="4" t="n"/>
-      <c r="J1720" s="2" t="n"/>
+      <c r="J1720" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1721">
       <c r="A1721" s="7" t="n"/>
@@ -45250,7 +45670,11 @@
           <t>Uyarı mesajı görüntülenmeli, ürün kaydedilmemelidir</t>
         </is>
       </c>
-      <c r="I1739" s="4" t="n"/>
+      <c r="I1739" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1739" s="8" t="n"/>
     </row>
     <row r="1741">
@@ -45347,7 +45771,11 @@
         </is>
       </c>
       <c r="I1742" s="4" t="n"/>
-      <c r="J1742" s="2" t="n"/>
+      <c r="J1742" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1743">
       <c r="A1743" s="7" t="n"/>
@@ -45800,7 +46228,11 @@
           <t>Uyarı mesajı görüntülenmeli, ürün kaydedilmemelidir</t>
         </is>
       </c>
-      <c r="I1761" s="4" t="n"/>
+      <c r="I1761" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1761" s="8" t="n"/>
     </row>
     <row r="1763">
@@ -45897,7 +46329,11 @@
         </is>
       </c>
       <c r="I1764" s="4" t="n"/>
-      <c r="J1764" s="2" t="n"/>
+      <c r="J1764" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1765">
       <c r="A1765" s="7" t="n"/>
@@ -46350,7 +46786,11 @@
           <t>Uyarı mesajı görüntülenmeli, ürün kaydedilmemelidir</t>
         </is>
       </c>
-      <c r="I1783" s="4" t="n"/>
+      <c r="I1783" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1783" s="8" t="n"/>
     </row>
     <row r="1785">
@@ -46447,7 +46887,11 @@
         </is>
       </c>
       <c r="I1786" s="4" t="n"/>
-      <c r="J1786" s="2" t="n"/>
+      <c r="J1786" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1787">
       <c r="A1787" s="7" t="n"/>
@@ -46900,7 +47344,11 @@
           <t>Uyarı mesajı görüntülenmeli, ürün kaydedilmemelidir</t>
         </is>
       </c>
-      <c r="I1805" s="4" t="n"/>
+      <c r="I1805" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1805" s="8" t="n"/>
     </row>
     <row r="1807">
@@ -46997,7 +47445,11 @@
         </is>
       </c>
       <c r="I1808" s="4" t="n"/>
-      <c r="J1808" s="2" t="n"/>
+      <c r="J1808" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1809">
       <c r="A1809" s="7" t="n"/>
@@ -47476,7 +47928,11 @@
           <t>Seçilen ek kategoriye ait ilaveler (Soslar) görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1828" s="4" t="n"/>
+      <c r="I1828" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1828" s="8" t="n"/>
     </row>
     <row r="1830">
@@ -47573,7 +48029,11 @@
         </is>
       </c>
       <c r="I1831" s="4" t="n"/>
-      <c r="J1831" s="2" t="n"/>
+      <c r="J1831" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1832">
       <c r="A1832" s="7" t="n"/>
@@ -48030,7 +48490,11 @@
           <t>Uyarı mesajı görüntülenmeli, ürün kaydedilmemelidir</t>
         </is>
       </c>
-      <c r="I1850" s="4" t="n"/>
+      <c r="I1850" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1850" s="8" t="n"/>
     </row>
     <row r="1852">
@@ -48127,7 +48591,11 @@
         </is>
       </c>
       <c r="I1853" s="4" t="n"/>
-      <c r="J1853" s="2" t="n"/>
+      <c r="J1853" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1854">
       <c r="A1854" s="7" t="n"/>
@@ -48584,7 +49052,11 @@
           <t>Uyarı mesajı görüntülenmeli, ürün kaydedilmemelidir</t>
         </is>
       </c>
-      <c r="I1872" s="4" t="n"/>
+      <c r="I1872" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1872" s="8" t="n"/>
     </row>
     <row r="1874">
@@ -48681,7 +49153,11 @@
         </is>
       </c>
       <c r="I1875" s="4" t="n"/>
-      <c r="J1875" s="2" t="n"/>
+      <c r="J1875" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1876">
       <c r="A1876" s="7" t="n"/>
@@ -49160,7 +49636,11 @@
           <t>Yüklenen resim ürün kartında görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1895" s="4" t="n"/>
+      <c r="I1895" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1895" s="8" t="n"/>
     </row>
     <row r="1897">
@@ -49257,7 +49737,11 @@
         </is>
       </c>
       <c r="I1898" s="4" t="n"/>
-      <c r="J1898" s="2" t="n"/>
+      <c r="J1898" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1899">
       <c r="A1899" s="7" t="n"/>
@@ -49740,7 +50224,11 @@
           <t>Ürün listelenmelidir</t>
         </is>
       </c>
-      <c r="I1918" s="4" t="n"/>
+      <c r="I1918" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1918" s="8" t="n"/>
     </row>
     <row r="1920">
@@ -49838,7 +50326,11 @@
         </is>
       </c>
       <c r="I1921" s="4" t="n"/>
-      <c r="J1921" s="2" t="n"/>
+      <c r="J1921" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1922">
       <c r="A1922" s="7" t="n"/>
@@ -50299,7 +50791,11 @@
           <t>Başarı mesajı görüntülenmeli, ürün listede güncel bilgilerle görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1940" s="4" t="n"/>
+      <c r="I1940" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1940" s="8" t="n"/>
     </row>
     <row r="1942">
@@ -50397,7 +50893,11 @@
         </is>
       </c>
       <c r="I1943" s="4" t="n"/>
-      <c r="J1943" s="2" t="n"/>
+      <c r="J1943" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1944">
       <c r="A1944" s="7" t="n"/>
@@ -50706,7 +51206,11 @@
           <t>Başarı mesajı görüntülenmeli, ürün listede güncel bilgilerle görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1956" s="4" t="n"/>
+      <c r="I1956" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1956" s="8" t="n"/>
     </row>
     <row r="1958">
@@ -50804,7 +51308,11 @@
         </is>
       </c>
       <c r="I1959" s="4" t="n"/>
-      <c r="J1959" s="2" t="n"/>
+      <c r="J1959" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1960">
       <c r="A1960" s="7" t="n"/>
@@ -51087,7 +51595,11 @@
           <t>Başarı mesajı görüntülenmeli, ürün listede güncel bilgilerle görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1971" s="4" t="n"/>
+      <c r="I1971" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1971" s="8" t="n"/>
     </row>
     <row r="1973">
@@ -51185,7 +51697,11 @@
         </is>
       </c>
       <c r="I1974" s="4" t="n"/>
-      <c r="J1974" s="2" t="n"/>
+      <c r="J1974" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1975">
       <c r="A1975" s="7" t="n"/>
@@ -51442,7 +51958,11 @@
           <t>Başarı mesajı görüntülenmeli, ürün listede güncel bilgilerle görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1985" s="4" t="n"/>
+      <c r="I1985" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1985" s="8" t="n"/>
     </row>
     <row r="1987">
@@ -51540,7 +52060,11 @@
         </is>
       </c>
       <c r="I1988" s="4" t="n"/>
-      <c r="J1988" s="2" t="n"/>
+      <c r="J1988" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="1989">
       <c r="A1989" s="7" t="n"/>
@@ -51797,7 +52321,11 @@
           <t>Başarı mesajı görüntülenmeli, ürün listede güncel bilgilerle görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I1999" s="4" t="n"/>
+      <c r="I1999" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J1999" s="8" t="n"/>
     </row>
     <row r="2001">
@@ -51895,7 +52423,11 @@
         </is>
       </c>
       <c r="I2002" s="4" t="n"/>
-      <c r="J2002" s="2" t="n"/>
+      <c r="J2002" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2003">
       <c r="A2003" s="7" t="n"/>
@@ -52152,7 +52684,11 @@
           <t>Başarı mesajı görüntülenmeli, ürün listede güncel bilgilerle görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I2013" s="4" t="n"/>
+      <c r="I2013" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2013" s="8" t="n"/>
     </row>
     <row r="2015">
@@ -52250,7 +52786,11 @@
         </is>
       </c>
       <c r="I2016" s="4" t="n"/>
-      <c r="J2016" s="2" t="n"/>
+      <c r="J2016" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2017">
       <c r="A2017" s="7" t="n"/>
@@ -52503,7 +53043,11 @@
           <t>Başarı mesajı görüntülenmeli, ürün listede güncel bilgilerle görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I2027" s="4" t="n"/>
+      <c r="I2027" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2027" s="8" t="n"/>
     </row>
     <row r="2029">
@@ -52601,7 +53145,11 @@
         </is>
       </c>
       <c r="I2030" s="4" t="n"/>
-      <c r="J2030" s="2" t="n"/>
+      <c r="J2030" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2031">
       <c r="A2031" s="7" t="n"/>
@@ -52854,7 +53402,11 @@
           <t>Uyarı mesajı görüntülenmeli, ürün güncellenmemelidir</t>
         </is>
       </c>
-      <c r="I2041" s="4" t="n"/>
+      <c r="I2041" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2041" s="8" t="n"/>
     </row>
     <row r="2043">
@@ -52952,7 +53504,11 @@
         </is>
       </c>
       <c r="I2044" s="4" t="n"/>
-      <c r="J2044" s="2" t="n"/>
+      <c r="J2044" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2045">
       <c r="A2045" s="7" t="n"/>
@@ -53209,7 +53765,11 @@
           <t>Ürün kullanıcı tarafında listelenmemelidir</t>
         </is>
       </c>
-      <c r="I2055" s="4" t="n"/>
+      <c r="I2055" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2055" s="8" t="n"/>
     </row>
     <row r="2057">
@@ -53307,7 +53867,11 @@
         </is>
       </c>
       <c r="I2058" s="4" t="n"/>
-      <c r="J2058" s="2" t="n"/>
+      <c r="J2058" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2059">
       <c r="A2059" s="7" t="n"/>
@@ -53516,7 +54080,11 @@
           <t>Başarı mesajı görüntülenmeli, ürün listeden kaldırılmalıdır</t>
         </is>
       </c>
-      <c r="I2067" s="4" t="n"/>
+      <c r="I2067" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2067" s="8" t="n"/>
     </row>
     <row r="2069">
@@ -53614,7 +54182,11 @@
         </is>
       </c>
       <c r="I2070" s="4" t="n"/>
-      <c r="J2070" s="2" t="n"/>
+      <c r="J2070" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2071">
       <c r="A2071" s="7" t="n"/>
@@ -53823,7 +54395,11 @@
           <t>Ürün silinmemeli, listede kalmalıdır</t>
         </is>
       </c>
-      <c r="I2079" s="4" t="n"/>
+      <c r="I2079" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2079" s="8" t="n"/>
     </row>
     <row r="2081">
@@ -53921,7 +54497,11 @@
         </is>
       </c>
       <c r="I2082" s="4" t="n"/>
-      <c r="J2082" s="2" t="n"/>
+      <c r="J2082" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2083">
       <c r="A2083" s="7" t="n"/>
@@ -54178,7 +54758,11 @@
           <t>Ürün listelenmelidir</t>
         </is>
       </c>
-      <c r="I2093" s="4" t="n"/>
+      <c r="I2093" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2093" s="8" t="n"/>
     </row>
     <row r="2095">
@@ -54275,7 +54859,11 @@
         </is>
       </c>
       <c r="I2096" s="4" t="n"/>
-      <c r="J2096" s="2" t="n"/>
+      <c r="J2096" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2097">
       <c r="A2097" s="7" t="n"/>
@@ -54458,7 +55046,11 @@
           <t>Kategori listesi (ad, açıklama, aktiflik durumu) görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I2104" s="4" t="n"/>
+      <c r="I2104" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2104" s="8" t="n"/>
     </row>
     <row r="2106">
@@ -54555,7 +55147,11 @@
         </is>
       </c>
       <c r="I2107" s="4" t="n"/>
-      <c r="J2107" s="2" t="n"/>
+      <c r="J2107" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2108">
       <c r="A2108" s="7" t="n"/>
@@ -54738,7 +55334,11 @@
           <t>Aktif kategoriler Active olarak işaretli görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I2115" s="4" t="n"/>
+      <c r="I2115" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2115" s="8" t="n"/>
     </row>
     <row r="2117">
@@ -54835,7 +55435,11 @@
         </is>
       </c>
       <c r="I2118" s="4" t="n"/>
-      <c r="J2118" s="2" t="n"/>
+      <c r="J2118" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2119">
       <c r="A2119" s="7" t="n"/>
@@ -55092,7 +55696,11 @@
           <t>Başarı mesajı görüntülenmeli, kategori listede görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I2129" s="4" t="n"/>
+      <c r="I2129" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2129" s="8" t="n"/>
     </row>
     <row r="2131">
@@ -55189,7 +55797,11 @@
         </is>
       </c>
       <c r="I2132" s="4" t="n"/>
-      <c r="J2132" s="2" t="n"/>
+      <c r="J2132" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2133">
       <c r="A2133" s="7" t="n"/>
@@ -55394,7 +56006,11 @@
           <t>Uyarı mesajı görüntülenmeli, kategori eklenmemelidir</t>
         </is>
       </c>
-      <c r="I2141" s="4" t="n"/>
+      <c r="I2141" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2141" s="8" t="n"/>
     </row>
     <row r="2143">
@@ -55492,7 +56108,11 @@
         </is>
       </c>
       <c r="I2144" s="4" t="n"/>
-      <c r="J2144" s="2" t="n"/>
+      <c r="J2144" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2145">
       <c r="A2145" s="7" t="n"/>
@@ -55701,7 +56321,11 @@
           <t>Başarı mesajı görüntülenmeli, kategori listeden kaldırılmalıdır</t>
         </is>
       </c>
-      <c r="I2153" s="4" t="n"/>
+      <c r="I2153" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2153" s="8" t="n"/>
     </row>
     <row r="2155">
@@ -55799,7 +56423,11 @@
         </is>
       </c>
       <c r="I2156" s="4" t="n"/>
-      <c r="J2156" s="2" t="n"/>
+      <c r="J2156" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2157">
       <c r="A2157" s="7" t="n"/>
@@ -56008,7 +56636,11 @@
           <t>Kategori silinmeli VEYA ürün bağlıysa silinemeyeceğine dair uyarı görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I2165" s="4" t="n"/>
+      <c r="I2165" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2165" s="8" t="n"/>
     </row>
     <row r="2167">
@@ -56105,7 +56737,11 @@
         </is>
       </c>
       <c r="I2168" s="4" t="n"/>
-      <c r="J2168" s="2" t="n"/>
+      <c r="J2168" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2169">
       <c r="A2169" s="7" t="n"/>
@@ -56288,7 +56924,11 @@
           <t>Ödeme listesi görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I2176" s="4" t="n"/>
+      <c r="I2176" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2176" s="8" t="n"/>
     </row>
     <row r="2178">
@@ -56385,7 +57025,11 @@
         </is>
       </c>
       <c r="I2179" s="4" t="n"/>
-      <c r="J2179" s="2" t="n"/>
+      <c r="J2179" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2180">
       <c r="A2180" s="7" t="n"/>
@@ -56590,7 +57234,11 @@
           <t>Diğer ödemeler listelenmelidir</t>
         </is>
       </c>
-      <c r="I2188" s="4" t="n"/>
+      <c r="I2188" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2188" s="8" t="n"/>
     </row>
     <row r="2190">
@@ -56687,7 +57335,11 @@
         </is>
       </c>
       <c r="I2191" s="4" t="n"/>
-      <c r="J2191" s="2" t="n"/>
+      <c r="J2191" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2192">
       <c r="A2192" s="7" t="n"/>
@@ -56958,7 +57610,11 @@
           <t>Ödeme statüsü görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I2203" s="4" t="n"/>
+      <c r="I2203" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2203" s="8" t="n"/>
     </row>
     <row r="2205">
@@ -57056,7 +57712,11 @@
         </is>
       </c>
       <c r="I2206" s="4" t="n"/>
-      <c r="J2206" s="2" t="n"/>
+      <c r="J2206" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2207">
       <c r="A2207" s="7" t="n"/>
@@ -57243,7 +57903,11 @@
           <t>Ödeme, siparişteki tutar ve ödeme yöntemi ile görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I2214" s="4" t="n"/>
+      <c r="I2214" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2214" s="8" t="n"/>
     </row>
     <row r="2216">
@@ -57340,7 +58004,11 @@
         </is>
       </c>
       <c r="I2217" s="4" t="n"/>
-      <c r="J2217" s="2" t="n"/>
+      <c r="J2217" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2218">
       <c r="A2218" s="7" t="n"/>
@@ -57523,7 +58191,11 @@
           <t>Ek kategori listesi görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I2225" s="4" t="n"/>
+      <c r="I2225" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2225" s="8" t="n"/>
     </row>
     <row r="2227">
@@ -57620,7 +58292,11 @@
         </is>
       </c>
       <c r="I2228" s="4" t="n"/>
-      <c r="J2228" s="2" t="n"/>
+      <c r="J2228" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2229">
       <c r="A2229" s="7" t="n"/>
@@ -57803,7 +58479,11 @@
           <t>Tüm ek kategoriler (ör. Soslar) ve ilaveler listelenmelidir</t>
         </is>
       </c>
-      <c r="I2236" s="4" t="n"/>
+      <c r="I2236" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2236" s="8" t="n"/>
     </row>
     <row r="2238">
@@ -57900,7 +58580,11 @@
         </is>
       </c>
       <c r="I2239" s="4" t="n"/>
-      <c r="J2239" s="2" t="n"/>
+      <c r="J2239" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2240">
       <c r="A2240" s="7" t="n"/>
@@ -58083,7 +58767,11 @@
           <t>Name, Description, Price ve Addition Category bilgileri görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I2247" s="4" t="n"/>
+      <c r="I2247" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2247" s="8" t="n"/>
     </row>
     <row r="2249">
@@ -58180,7 +58868,11 @@
         </is>
       </c>
       <c r="I2250" s="4" t="n"/>
-      <c r="J2250" s="2" t="n"/>
+      <c r="J2250" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2251">
       <c r="A2251" s="7" t="n"/>
@@ -58489,7 +59181,11 @@
           <t>Başarı mesajı görüntülenmeli, kayıt listede görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I2263" s="4" t="n"/>
+      <c r="I2263" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2263" s="8" t="n"/>
     </row>
     <row r="2265">
@@ -58586,7 +59282,11 @@
         </is>
       </c>
       <c r="I2266" s="4" t="n"/>
-      <c r="J2266" s="2" t="n"/>
+      <c r="J2266" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2267">
       <c r="A2267" s="7" t="n"/>
@@ -58891,7 +59591,11 @@
           <t>Uyarı mesajı görüntülenmeli, kayıt eklenmemelidir</t>
         </is>
       </c>
-      <c r="I2279" s="4" t="n"/>
+      <c r="I2279" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2279" s="8" t="n"/>
     </row>
     <row r="2281">
@@ -58988,7 +59692,11 @@
         </is>
       </c>
       <c r="I2282" s="4" t="n"/>
-      <c r="J2282" s="2" t="n"/>
+      <c r="J2282" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2283">
       <c r="A2283" s="7" t="n"/>
@@ -59293,7 +60001,11 @@
           <t>Uyarı mesajı görüntülenmeli, kayıt eklenmemelidir</t>
         </is>
       </c>
-      <c r="I2295" s="4" t="n"/>
+      <c r="I2295" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2295" s="8" t="n"/>
     </row>
     <row r="2297">
@@ -59390,7 +60102,11 @@
         </is>
       </c>
       <c r="I2298" s="4" t="n"/>
-      <c r="J2298" s="2" t="n"/>
+      <c r="J2298" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2299">
       <c r="A2299" s="7" t="n"/>
@@ -59695,7 +60411,11 @@
           <t>Uyarı mesajı görüntülenmeli, kayıt eklenmemelidir</t>
         </is>
       </c>
-      <c r="I2311" s="4" t="n"/>
+      <c r="I2311" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2311" s="8" t="n"/>
     </row>
     <row r="2313">
@@ -59792,7 +60512,11 @@
         </is>
       </c>
       <c r="I2314" s="4" t="n"/>
-      <c r="J2314" s="2" t="n"/>
+      <c r="J2314" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2315">
       <c r="A2315" s="7" t="n"/>
@@ -60097,7 +60821,11 @@
           <t>Uyarı mesajı görüntülenmeli, kayıt eklenmemelidir</t>
         </is>
       </c>
-      <c r="I2327" s="4" t="n"/>
+      <c r="I2327" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2327" s="8" t="n"/>
     </row>
     <row r="2329">
@@ -60194,7 +60922,11 @@
         </is>
       </c>
       <c r="I2330" s="4" t="n"/>
-      <c r="J2330" s="2" t="n"/>
+      <c r="J2330" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2331">
       <c r="A2331" s="7" t="n"/>
@@ -60473,7 +61205,11 @@
           <t>Uyarı mesajı görüntülenmeli, kayıt eklenmemelidir</t>
         </is>
       </c>
-      <c r="I2342" s="4" t="n"/>
+      <c r="I2342" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2342" s="8" t="n"/>
     </row>
     <row r="2344">
@@ -60571,7 +61307,11 @@
         </is>
       </c>
       <c r="I2345" s="4" t="n"/>
-      <c r="J2345" s="2" t="n"/>
+      <c r="J2345" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2346">
       <c r="A2346" s="7" t="n"/>
@@ -60780,7 +61520,11 @@
           <t>Başarı mesajı görüntülenmeli, kayıt listeden kaldırılmalıdır</t>
         </is>
       </c>
-      <c r="I2354" s="4" t="n"/>
+      <c r="I2354" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2354" s="8" t="n"/>
     </row>
     <row r="2356">
@@ -62800,7 +63544,11 @@
         </is>
       </c>
       <c r="I2431" s="4" t="n"/>
-      <c r="J2431" s="2" t="n"/>
+      <c r="J2431" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2432">
       <c r="A2432" s="7" t="n"/>
@@ -63021,7 +63769,11 @@
           <t>Mesaj Name, Email, Subject ve Message bilgileri ile listelenmelidir</t>
         </is>
       </c>
-      <c r="I2440" s="4" t="n"/>
+      <c r="I2440" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2440" s="8" t="n"/>
     </row>
     <row r="2442">
@@ -63119,7 +63871,11 @@
         </is>
       </c>
       <c r="I2443" s="4" t="n"/>
-      <c r="J2443" s="2" t="n"/>
+      <c r="J2443" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2444">
       <c r="A2444" s="7" t="n"/>
@@ -63302,7 +64058,11 @@
           <t>Tüm mesajlar Name, Email, Subject ve Date bilgileri ile listelenmelidir</t>
         </is>
       </c>
-      <c r="I2451" s="4" t="n"/>
+      <c r="I2451" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2451" s="8" t="n"/>
     </row>
     <row r="2453">
@@ -63400,7 +64160,11 @@
         </is>
       </c>
       <c r="I2454" s="4" t="n"/>
-      <c r="J2454" s="2" t="n"/>
+      <c r="J2454" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2455">
       <c r="A2455" s="7" t="n"/>
@@ -63605,7 +64369,11 @@
           <t>Mesajın tam içeriği görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I2463" s="4" t="n"/>
+      <c r="I2463" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2463" s="8" t="n"/>
     </row>
     <row r="2465">
@@ -63703,7 +64471,11 @@
         </is>
       </c>
       <c r="I2466" s="4" t="n"/>
-      <c r="J2466" s="2" t="n"/>
+      <c r="J2466" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2467">
       <c r="A2467" s="7" t="n"/>
@@ -63912,7 +64684,11 @@
           <t>Tüm mesajlar listelenmelidir</t>
         </is>
       </c>
-      <c r="I2475" s="4" t="n"/>
+      <c r="I2475" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2475" s="8" t="n"/>
     </row>
     <row r="2477">
@@ -64010,7 +64786,11 @@
         </is>
       </c>
       <c r="I2478" s="4" t="n"/>
-      <c r="J2478" s="2" t="n"/>
+      <c r="J2478" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2479">
       <c r="A2479" s="7" t="n"/>
@@ -64245,7 +65025,11 @@
           <t>Yalnızca Email kriterine uyan mesajlar listelenmelidir</t>
         </is>
       </c>
-      <c r="I2488" s="4" t="n"/>
+      <c r="I2488" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2488" s="8" t="n"/>
     </row>
     <row r="2490">
@@ -64343,7 +65127,11 @@
         </is>
       </c>
       <c r="I2491" s="4" t="n"/>
-      <c r="J2491" s="2" t="n"/>
+      <c r="J2491" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2492">
       <c r="A2492" s="7" t="n"/>
@@ -64578,7 +65366,11 @@
           <t>Yalnızca Subject kriterine uyan mesajlar listelenmelidir</t>
         </is>
       </c>
-      <c r="I2501" s="4" t="n"/>
+      <c r="I2501" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2501" s="8" t="n"/>
     </row>
     <row r="2503">
@@ -64676,7 +65468,11 @@
         </is>
       </c>
       <c r="I2504" s="4" t="n"/>
-      <c r="J2504" s="2" t="n"/>
+      <c r="J2504" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2505">
       <c r="A2505" s="7" t="n"/>
@@ -64911,7 +65707,11 @@
           <t>Yalnızca Date kriterine uyan mesajlar listelenmelidir</t>
         </is>
       </c>
-      <c r="I2514" s="4" t="n"/>
+      <c r="I2514" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2514" s="8" t="n"/>
     </row>
     <row r="2516">
@@ -65009,7 +65809,11 @@
         </is>
       </c>
       <c r="I2517" s="4" t="n"/>
-      <c r="J2517" s="2" t="n"/>
+      <c r="J2517" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2518">
       <c r="A2518" s="7" t="n"/>
@@ -65244,7 +66048,11 @@
           <t>Yalnızca Time kriterine uyan mesajlar listelenmelidir</t>
         </is>
       </c>
-      <c r="I2527" s="4" t="n"/>
+      <c r="I2527" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2527" s="8" t="n"/>
     </row>
     <row r="2529">
@@ -65342,7 +66150,11 @@
         </is>
       </c>
       <c r="I2530" s="4" t="n"/>
-      <c r="J2530" s="2" t="n"/>
+      <c r="J2530" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2531">
       <c r="A2531" s="7" t="n"/>
@@ -65551,7 +66363,11 @@
           <t>Mesaj listelenmemeli, bilgilendirme görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I2539" s="4" t="n"/>
+      <c r="I2539" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2539" s="8" t="n"/>
     </row>
     <row r="2541">
@@ -65649,7 +66465,11 @@
         </is>
       </c>
       <c r="I2542" s="4" t="n"/>
-      <c r="J2542" s="2" t="n"/>
+      <c r="J2542" s="11" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
     </row>
     <row r="2543">
       <c r="A2543" s="7" t="n"/>
@@ -65854,7 +66674,11 @@
           <t>Başarı mesajı görüntülenmeli, mesaj listeden kaldırılmalıdır</t>
         </is>
       </c>
-      <c r="I2551" s="4" t="n"/>
+      <c r="I2551" s="4" t="inlineStr">
+        <is>
+          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+        </is>
+      </c>
       <c r="J2551" s="8" t="n"/>
     </row>
   </sheetData>
@@ -67024,10 +67848,10 @@
         <v>0</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -67067,10 +67891,10 @@
         <v>0</v>
       </c>
       <c r="J5" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="K5" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="K5" s="4" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -67325,10 +68149,10 @@
         <v>0</v>
       </c>
       <c r="J11" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K11" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="K11" s="4" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -67368,10 +68192,10 @@
         <v>0</v>
       </c>
       <c r="J12" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K12" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="K12" s="4" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -67411,10 +68235,10 @@
         <v>0</v>
       </c>
       <c r="J13" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K13" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="K13" s="4" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -67454,10 +68278,10 @@
         <v>0</v>
       </c>
       <c r="J14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K14" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="K14" s="4" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -67497,10 +68321,10 @@
         <v>0</v>
       </c>
       <c r="J15" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="K15" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="K15" s="4" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="16">
@@ -67540,10 +68364,10 @@
         <v>0</v>
       </c>
       <c r="J16" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="K16" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="K16" s="4" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="17">
@@ -67583,10 +68407,10 @@
         <v>0</v>
       </c>
       <c r="J17" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K17" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="K17" s="4" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="18">
@@ -67626,10 +68450,10 @@
         <v>0</v>
       </c>
       <c r="J18" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K18" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="K18" s="4" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="19">
@@ -67669,10 +68493,10 @@
         <v>0</v>
       </c>
       <c r="J19" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K19" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="K19" s="4" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="20">
@@ -67712,10 +68536,10 @@
         <v>0</v>
       </c>
       <c r="J20" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="K20" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="K20" s="4" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="21">
@@ -67755,10 +68579,10 @@
         <v>0</v>
       </c>
       <c r="J21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="K21" s="4" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -67798,10 +68622,10 @@
         <v>0</v>
       </c>
       <c r="J22" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="K22" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="K22" s="4" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="23">
@@ -67829,10 +68653,10 @@
         <v>29</v>
       </c>
       <c r="J23" s="12" t="n">
-        <v>4</v>
+        <v>107</v>
       </c>
       <c r="K23" s="12" t="n">
-        <v>106</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
Admin paneli manuel koşum sonuçları eklendi; SCRUM-257..269 bug kayıtları
Test case dosyası, Test Planı v1.1 (Test Özet Raporu) ve Xray execution
sonuç dosyası güncellendi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Snack_Attack_Test_Cases_Yildiray_Kosedag.xlsx
+++ b/docs/Snack_Attack_Test_Cases_Yildiray_Kosedag.xlsx
@@ -11360,7 +11360,7 @@
       </c>
       <c r="I418" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J418" s="8" t="n"/>
@@ -11908,7 +11908,7 @@
       </c>
       <c r="I440" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J440" s="8" t="n"/>
@@ -12456,7 +12456,7 @@
       </c>
       <c r="I462" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J462" s="8" t="n"/>
@@ -13004,7 +13004,7 @@
       </c>
       <c r="I484" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J484" s="8" t="n"/>
@@ -13552,7 +13552,7 @@
       </c>
       <c r="I506" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J506" s="8" t="n"/>
@@ -14100,7 +14100,7 @@
       </c>
       <c r="I528" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J528" s="8" t="n"/>
@@ -14648,7 +14648,7 @@
       </c>
       <c r="I550" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J550" s="8" t="n"/>
@@ -15196,7 +15196,7 @@
       </c>
       <c r="I572" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J572" s="8" t="n"/>
@@ -15748,7 +15748,7 @@
       </c>
       <c r="I594" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J594" s="8" t="n"/>
@@ -16300,7 +16300,7 @@
       </c>
       <c r="I616" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J616" s="8" t="n"/>
@@ -16852,7 +16852,7 @@
       </c>
       <c r="I638" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J638" s="8" t="n"/>
@@ -17404,7 +17404,7 @@
       </c>
       <c r="I660" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J660" s="8" t="n"/>
@@ -17956,7 +17956,7 @@
       </c>
       <c r="I682" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J682" s="8" t="n"/>
@@ -18508,7 +18508,7 @@
       </c>
       <c r="I704" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J704" s="8" t="n"/>
@@ -19056,7 +19056,7 @@
       </c>
       <c r="I726" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J726" s="8" t="n"/>
@@ -19604,7 +19604,7 @@
       </c>
       <c r="I748" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J748" s="8" t="n"/>
@@ -20156,7 +20156,7 @@
       </c>
       <c r="I770" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J770" s="8" t="n"/>
@@ -20707,7 +20707,7 @@
       </c>
       <c r="I792" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J792" s="8" t="n"/>
@@ -21033,7 +21033,7 @@
       </c>
       <c r="I805" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J805" s="8" t="n"/>
@@ -21277,7 +21277,7 @@
       </c>
       <c r="I814" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J814" s="8" t="n"/>
@@ -21506,7 +21506,7 @@
       </c>
       <c r="I823" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J823" s="8" t="n"/>
@@ -21728,7 +21728,7 @@
       </c>
       <c r="I831" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J831" s="8" t="n"/>
@@ -21946,7 +21946,7 @@
       </c>
       <c r="I839" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J839" s="8" t="n"/>
@@ -22138,7 +22138,7 @@
       </c>
       <c r="I846" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J846" s="8" t="n"/>
@@ -22334,7 +22334,7 @@
       </c>
       <c r="I853" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J853" s="8" t="n"/>
@@ -22530,7 +22530,7 @@
       </c>
       <c r="I860" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J860" s="8" t="n"/>
@@ -22752,7 +22752,7 @@
       </c>
       <c r="I868" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J868" s="8" t="n"/>
@@ -22973,7 +22973,7 @@
       </c>
       <c r="I876" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J876" s="8" t="n"/>
@@ -23146,7 +23146,7 @@
       </c>
       <c r="I882" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
         </is>
       </c>
       <c r="J882" s="8" t="n"/>
@@ -37354,9 +37354,9 @@
         </is>
       </c>
       <c r="I1417" s="4" t="n"/>
-      <c r="J1417" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1417" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -37569,7 +37569,7 @@
       </c>
       <c r="I1426" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Customer Management'ta User ID, First Name, Last Name, Email, Phone Number, Region Code kolonları ile 14 kullanıcı görüntülendi.</t>
         </is>
       </c>
       <c r="J1426" s="8" t="n"/>
@@ -37668,9 +37668,9 @@
         </is>
       </c>
       <c r="I1429" s="4" t="n"/>
-      <c r="J1429" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1429" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -37883,7 +37883,7 @@
       </c>
       <c r="I1438" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Tüm kullanıcılar listelendi, sayfalama mevcut. Not: telefon formatı tutarsız (+90532… / 541…).</t>
         </is>
       </c>
       <c r="J1438" s="8" t="n"/>
@@ -38220,7 +38220,7 @@
       </c>
       <c r="I1451" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
         </is>
       </c>
       <c r="J1451" s="8" t="n"/>
@@ -38534,7 +38534,7 @@
       </c>
       <c r="I1463" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
         </is>
       </c>
       <c r="J1463" s="8" t="n"/>
@@ -38709,7 +38709,7 @@
       </c>
       <c r="I1469" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
         </is>
       </c>
       <c r="J1469" s="8" t="n"/>
@@ -38808,9 +38808,9 @@
         </is>
       </c>
       <c r="I1472" s="4" t="n"/>
-      <c r="J1472" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1472" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -39023,7 +39023,7 @@
       </c>
       <c r="I1481" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Admin Management'ta mehmet@admin.com (7) ve admin@example.com (1) bilgileri görüntülendi.</t>
         </is>
       </c>
       <c r="J1481" s="8" t="n"/>
@@ -39122,9 +39122,9 @@
         </is>
       </c>
       <c r="I1484" s="4" t="n"/>
-      <c r="J1484" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1484" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -39337,7 +39337,7 @@
       </c>
       <c r="I1493" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Tüm adminler listelendi.</t>
         </is>
       </c>
       <c r="J1493" s="8" t="n"/>
@@ -39674,7 +39674,7 @@
       </c>
       <c r="I1506" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
         </is>
       </c>
       <c r="J1506" s="8" t="n"/>
@@ -39988,7 +39988,7 @@
       </c>
       <c r="I1518" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
         </is>
       </c>
       <c r="J1518" s="8" t="n"/>
@@ -40302,7 +40302,7 @@
       </c>
       <c r="I1530" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
         </is>
       </c>
       <c r="J1530" s="8" t="n"/>
@@ -40401,9 +40401,9 @@
         </is>
       </c>
       <c r="I1533" s="4" t="n"/>
-      <c r="J1533" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1533" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -40590,7 +40590,7 @@
       </c>
       <c r="I1541" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>ID, Name, Address, Total Price, Date, Status, Payment görüntülendi; ancak kullanıcı tarafında CANCELED olan Order #2 admin panelinde PENDING görünüyor, statü listesinde CANCELED seçeneği yok. (Bug: SCRUM-264)</t>
         </is>
       </c>
       <c r="J1541" s="8" t="n"/>
@@ -40689,9 +40689,9 @@
         </is>
       </c>
       <c r="I1544" s="4" t="n"/>
-      <c r="J1544" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1544" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -40900,7 +40900,7 @@
       </c>
       <c r="I1553" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Siparişler listelendi (Order #2).</t>
         </is>
       </c>
       <c r="J1553" s="8" t="n"/>
@@ -40999,9 +40999,9 @@
         </is>
       </c>
       <c r="I1556" s="4" t="n"/>
-      <c r="J1556" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1556" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -41210,7 +41210,7 @@
       </c>
       <c r="I1565" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Sipariş satırında detay görüntüleme butonu/aksiyonu yok; sipariş detayı açılamıyor. (Bug: SCRUM-267)</t>
         </is>
       </c>
       <c r="J1565" s="8" t="n"/>
@@ -41547,7 +41547,7 @@
       </c>
       <c r="I1578" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
         </is>
       </c>
       <c r="J1578" s="8" t="n"/>
@@ -41884,7 +41884,7 @@
       </c>
       <c r="I1591" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
         </is>
       </c>
       <c r="J1591" s="8" t="n"/>
@@ -42199,7 +42199,7 @@
       </c>
       <c r="I1603" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak. Not: CANCELED Order #2'nin statü dropdown'ı aktif görünüyor. (Bug: SCRUM-264)</t>
         </is>
       </c>
       <c r="J1603" s="8" t="n"/>
@@ -42298,9 +42298,9 @@
         </is>
       </c>
       <c r="I1606" s="4" t="n"/>
-      <c r="J1606" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1606" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -42487,7 +42487,7 @@
       </c>
       <c r="I1614" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Product Management'ta ürünler ID, Image, Name, Description, Price, Order Count, Category, Created At ile görüntülendi (3 sayfa).</t>
         </is>
       </c>
       <c r="J1614" s="8" t="n"/>
@@ -42586,9 +42586,9 @@
         </is>
       </c>
       <c r="I1617" s="4" t="n"/>
-      <c r="J1617" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1617" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -42801,7 +42801,7 @@
       </c>
       <c r="I1626" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Ürünler sayfalama ile listelendi. Not: tüm ürünlerde Order Count = 35.</t>
         </is>
       </c>
       <c r="J1626" s="8" t="n"/>
@@ -42900,9 +42900,9 @@
         </is>
       </c>
       <c r="I1629" s="4" t="n"/>
-      <c r="J1629" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1629" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -43115,7 +43115,7 @@
       </c>
       <c r="I1638" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>"QA test urunu" araması → yalnızca eşleşen test ürünleri listelendi.</t>
         </is>
       </c>
       <c r="J1638" s="8" t="n"/>
@@ -43214,9 +43214,9 @@
         </is>
       </c>
       <c r="I1641" s="4" t="n"/>
-      <c r="J1641" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1641" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -43429,7 +43429,7 @@
       </c>
       <c r="I1650" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>"zzqxyokurun" araması → ürün listelenmedi. Not: bilgilendirme mesajı yok.</t>
         </is>
       </c>
       <c r="J1650" s="8" t="n"/>
@@ -43528,9 +43528,9 @@
         </is>
       </c>
       <c r="I1653" s="4" t="n"/>
-      <c r="J1653" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1653" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -43991,7 +43991,7 @@
       </c>
       <c r="I1672" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>"QA YK Tam Urun" (100, indirim 10, HAMBURGER, Soslar, resim) → "Ürün başarıyla oluşturuldu!"; listede ve kullanıcı Products sayfasında görüntülendi. Not: indirim fiyata yansımıyor.</t>
         </is>
       </c>
       <c r="J1672" s="8" t="n"/>
@@ -44097,9 +44097,9 @@
         </is>
       </c>
       <c r="I1676" s="4" t="n"/>
-      <c r="J1676" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1676" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -44556,7 +44556,7 @@
       </c>
       <c r="I1695" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>İndirim alanına dokunulmadan "QA YK Kategorisiz" eklendi, "Ürün başarıyla oluşturuldu!" görüntülendi.</t>
         </is>
       </c>
       <c r="J1695" s="8" t="n"/>
@@ -44655,9 +44655,9 @@
         </is>
       </c>
       <c r="I1698" s="4" t="n"/>
-      <c r="J1698" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1698" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -45114,7 +45114,7 @@
       </c>
       <c r="I1717" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Name boş → "Lütfen bu alanı doldurun." uyarısı görüntülendi, ürün eklenmedi.</t>
         </is>
       </c>
       <c r="J1717" s="8" t="n"/>
@@ -45213,9 +45213,9 @@
         </is>
       </c>
       <c r="I1720" s="4" t="n"/>
-      <c r="J1720" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1720" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -45672,7 +45672,7 @@
       </c>
       <c r="I1739" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Description boş → "Lütfen bu alanı doldurun." uyarısı görüntülendi, ürün eklenmedi.</t>
         </is>
       </c>
       <c r="J1739" s="8" t="n"/>
@@ -45771,9 +45771,9 @@
         </is>
       </c>
       <c r="I1742" s="4" t="n"/>
-      <c r="J1742" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1742" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -46230,7 +46230,7 @@
       </c>
       <c r="I1761" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Contents boş → "Lütfen bu alanı doldurun." uyarısı görüntülendi, ürün eklenmedi.</t>
         </is>
       </c>
       <c r="J1761" s="8" t="n"/>
@@ -46329,9 +46329,9 @@
         </is>
       </c>
       <c r="I1764" s="4" t="n"/>
-      <c r="J1764" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1764" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -46788,7 +46788,7 @@
       </c>
       <c r="I1783" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Price boş → "Lütfen bu alanı doldurun." uyarısı görüntülendi, ürün eklenmedi.</t>
         </is>
       </c>
       <c r="J1783" s="8" t="n"/>
@@ -46887,9 +46887,9 @@
         </is>
       </c>
       <c r="I1786" s="4" t="n"/>
-      <c r="J1786" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1786" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -47346,7 +47346,7 @@
       </c>
       <c r="I1805" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Kategori seçilmeden Create Product → "Ürün başarıyla oluşturuldu!"; ürün kategorisiz olarak kullanıcı tarafında listeleniyor. (Bug: SCRUM-258)</t>
         </is>
       </c>
       <c r="J1805" s="8" t="n"/>
@@ -47445,9 +47445,9 @@
         </is>
       </c>
       <c r="I1808" s="4" t="n"/>
-      <c r="J1808" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1808" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -47930,7 +47930,7 @@
       </c>
       <c r="I1828" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Soslar seçilen ürünün kullanıcı detayında Karışık Sos, Ketçap, Mayonez, Acı Sos, Special Sos, Hardal Sosu (+₺5.00) görüntülendi.</t>
         </is>
       </c>
       <c r="J1828" s="8" t="n"/>
@@ -48029,9 +48029,9 @@
         </is>
       </c>
       <c r="I1831" s="4" t="n"/>
-      <c r="J1831" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1831" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -48492,7 +48492,7 @@
       </c>
       <c r="I1850" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Price = -10 → "Lütfen tüm zorunlu alanları doldurun!" uyarısı, ürün eklenmedi. Not: mesaj yanıltıcı.</t>
         </is>
       </c>
       <c r="J1850" s="8" t="n"/>
@@ -48591,9 +48591,9 @@
         </is>
       </c>
       <c r="I1853" s="4" t="n"/>
-      <c r="J1853" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1853" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -49054,7 +49054,7 @@
       </c>
       <c r="I1872" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Price 50 / Discount 150 → "Ürün başarıyla oluşturuldu!"; indirimi fiyattan büyük ürün kaydedildi. (Bug: SCRUM-259)</t>
         </is>
       </c>
       <c r="J1872" s="8" t="n"/>
@@ -49153,9 +49153,9 @@
         </is>
       </c>
       <c r="I1875" s="4" t="n"/>
-      <c r="J1875" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1875" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -49638,7 +49638,7 @@
       </c>
       <c r="I1895" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Yüklenen resim önizlemede, ürün kartında ve detayda görüntülendi.</t>
         </is>
       </c>
       <c r="J1895" s="8" t="n"/>
@@ -49737,9 +49737,9 @@
         </is>
       </c>
       <c r="I1898" s="4" t="n"/>
-      <c r="J1898" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1898" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -50226,7 +50226,7 @@
       </c>
       <c r="I1918" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Available ve Active işaretli eklenen ürün kullanıcı Products aramasında listelendi.</t>
         </is>
       </c>
       <c r="J1918" s="8" t="n"/>
@@ -50326,9 +50326,9 @@
         </is>
       </c>
       <c r="I1921" s="4" t="n"/>
-      <c r="J1921" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1921" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -50793,7 +50793,7 @@
       </c>
       <c r="I1940" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Ad, açıklama, içerik, fiyat 100→120, indirim 10→20, kategori HAMBURGER→PIZZA, ek Soslar→Mezeler ve resim güncellendi; kullanıcı tarafında tümü güncel görüntülendi.</t>
         </is>
       </c>
       <c r="J1940" s="8" t="n"/>
@@ -50893,9 +50893,9 @@
         </is>
       </c>
       <c r="I1943" s="4" t="n"/>
-      <c r="J1943" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1943" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -51208,7 +51208,7 @@
       </c>
       <c r="I1956" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Name, Description ve İçerik güncellendi, listede ve kullanıcı tarafında yeni değerler görüntülendi.</t>
         </is>
       </c>
       <c r="J1956" s="8" t="n"/>
@@ -51308,9 +51308,9 @@
         </is>
       </c>
       <c r="I1959" s="4" t="n"/>
-      <c r="J1959" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1959" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -51597,7 +51597,7 @@
       </c>
       <c r="I1971" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Fiyat 120 ve indirim 20 kaydedildi. Not: indirim kullanıcı tarafında fiyata yansımıyor.</t>
         </is>
       </c>
       <c r="J1971" s="8" t="n"/>
@@ -51697,9 +51697,9 @@
         </is>
       </c>
       <c r="I1974" s="4" t="n"/>
-      <c r="J1974" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1974" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -51960,7 +51960,7 @@
       </c>
       <c r="I1985" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Kategori PIZZA olarak güncellendi, kullanıcı kartında Pizza rozeti görüntülendi.</t>
         </is>
       </c>
       <c r="J1985" s="8" t="n"/>
@@ -52060,9 +52060,9 @@
         </is>
       </c>
       <c r="I1988" s="4" t="n"/>
-      <c r="J1988" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1988" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -52323,7 +52323,7 @@
       </c>
       <c r="I1999" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Ek kategori Mezeler oldu; detayda Acılı Ezme, Yoğun Baharatlı Ezme, Ekşili Ezme görüntülendi.</t>
         </is>
       </c>
       <c r="J1999" s="8" t="n"/>
@@ -52423,9 +52423,9 @@
         </is>
       </c>
       <c r="I2002" s="4" t="n"/>
-      <c r="J2002" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2002" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -52686,7 +52686,7 @@
       </c>
       <c r="I2013" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Yeni resim yüklendi, kart ve detayda yeni resim görüntülendi.</t>
         </is>
       </c>
       <c r="J2013" s="8" t="n"/>
@@ -52786,9 +52786,9 @@
         </is>
       </c>
       <c r="I2016" s="4" t="n"/>
-      <c r="J2016" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2016" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -53045,7 +53045,7 @@
       </c>
       <c r="I2027" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Ürün Düzenleme formunda yalnızca "Popüler mi?" ve "Mevcut mu?" var; Active seçeneği bulunmuyor, doğrulanamadı. Mevcut işaretli kaldı. (Bug: SCRUM-260)</t>
         </is>
       </c>
       <c r="J2027" s="8" t="n"/>
@@ -53145,9 +53145,9 @@
         </is>
       </c>
       <c r="I2030" s="4" t="n"/>
-      <c r="J2030" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2030" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -53404,7 +53404,7 @@
       </c>
       <c r="I2041" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Ürün Adı boş → "Lütfen bu alanı doldurun.", ürün güncellenmedi.</t>
         </is>
       </c>
       <c r="J2041" s="8" t="n"/>
@@ -53504,9 +53504,9 @@
         </is>
       </c>
       <c r="I2044" s="4" t="n"/>
-      <c r="J2044" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2044" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -53767,7 +53767,7 @@
       </c>
       <c r="I2055" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>"Mevcut mu?" kaldırılıp Güncelle → "Ürün başarıyla güncellendi!"; ürün kullanıcı aramasında listelenmedi.</t>
         </is>
       </c>
       <c r="J2055" s="8" t="n"/>
@@ -53867,9 +53867,9 @@
         </is>
       </c>
       <c r="I2058" s="4" t="n"/>
-      <c r="J2058" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2058" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -54082,7 +54082,7 @@
       </c>
       <c r="I2067" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Silme onaylandığında DELETE https://snackattack.deployedprojects.xyz/api/products/30 → 404; ürün silinmedi, hata mesajı gösterilmedi. (Bug: SCRUM-257)</t>
         </is>
       </c>
       <c r="J2067" s="8" t="n"/>
@@ -54182,9 +54182,9 @@
         </is>
       </c>
       <c r="I2070" s="4" t="n"/>
-      <c r="J2070" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2070" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -54397,7 +54397,7 @@
       </c>
       <c r="I2079" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Onay penceresi ("Are you sure you want to delete this product?") iptal edildi, ürün listede kaldı.</t>
         </is>
       </c>
       <c r="J2079" s="8" t="n"/>
@@ -54497,9 +54497,9 @@
         </is>
       </c>
       <c r="I2082" s="4" t="n"/>
-      <c r="J2082" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2082" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -54760,7 +54760,7 @@
       </c>
       <c r="I2093" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>"Mevcut mu?" tekrar işaretlendi → "Ürün başarıyla güncellendi!", ürün kullanıcı tarafında listelendi.</t>
         </is>
       </c>
       <c r="J2093" s="8" t="n"/>
@@ -54859,9 +54859,9 @@
         </is>
       </c>
       <c r="I2096" s="4" t="n"/>
-      <c r="J2096" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2096" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -55048,7 +55048,7 @@
       </c>
       <c r="I2104" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Category Management Panel: ID, Name, Active, Created At ile 6 kategori görüntülendi.</t>
         </is>
       </c>
       <c r="J2104" s="8" t="n"/>
@@ -55147,9 +55147,9 @@
         </is>
       </c>
       <c r="I2107" s="4" t="n"/>
-      <c r="J2107" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2107" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -55336,7 +55336,7 @@
       </c>
       <c r="I2115" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Tüm kategoriler Active ✓ olarak görüntülendi.</t>
         </is>
       </c>
       <c r="J2115" s="8" t="n"/>
@@ -55435,9 +55435,9 @@
         </is>
       </c>
       <c r="I2118" s="4" t="n"/>
-      <c r="J2118" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2118" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -55698,7 +55698,7 @@
       </c>
       <c r="I2129" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>"QAYKTEST" eklendi, listede görüntülendi (ID 7). Not: başarı mesajı görüntülenmedi.</t>
         </is>
       </c>
       <c r="J2129" s="8" t="n"/>
@@ -55797,9 +55797,9 @@
         </is>
       </c>
       <c r="I2132" s="4" t="n"/>
-      <c r="J2132" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2132" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -56008,7 +56008,7 @@
       </c>
       <c r="I2141" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Name boş → "Lütfen bu alanı doldurun.", kategori eklenmedi.</t>
         </is>
       </c>
       <c r="J2141" s="8" t="n"/>
@@ -56108,9 +56108,9 @@
         </is>
       </c>
       <c r="I2144" s="4" t="n"/>
-      <c r="J2144" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2144" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -56323,7 +56323,7 @@
       </c>
       <c r="I2153" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>"QAYKTEST" silindi, listeden kaldırıldı. Not: onay metni "delete this product?" (yanlış metin).</t>
         </is>
       </c>
       <c r="J2153" s="8" t="n"/>
@@ -56423,9 +56423,9 @@
         </is>
       </c>
       <c r="I2156" s="4" t="n"/>
-      <c r="J2156" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2156" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -56638,7 +56638,7 @@
       </c>
       <c r="I2165" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Ürün bağlı test kategorisi (QAYKBAGLI) silinmek istendi → sunucu 500 döndü, kategori silinmedi ve hiçbir uyarı görüntülenmedi. (Bug: SCRUM-266)</t>
         </is>
       </c>
       <c r="J2165" s="8" t="n"/>
@@ -56737,9 +56737,9 @@
         </is>
       </c>
       <c r="I2168" s="4" t="n"/>
-      <c r="J2168" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2168" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -56926,7 +56926,7 @@
       </c>
       <c r="I2176" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Payment Management paneli (Payment ID, Order ID, User ID, Amount, Payment Date) görüntülendi.</t>
         </is>
       </c>
       <c r="J2176" s="8" t="n"/>
@@ -57025,9 +57025,9 @@
         </is>
       </c>
       <c r="I2179" s="4" t="n"/>
-      <c r="J2179" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2179" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -57236,7 +57236,7 @@
       </c>
       <c r="I2188" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>"No payments found." – Order #2 (CASH, $75.00) için ödeme kaydı listelenmiyor. (Bug: SCRUM-265)</t>
         </is>
       </c>
       <c r="J2188" s="8" t="n"/>
@@ -57335,9 +57335,9 @@
         </is>
       </c>
       <c r="I2191" s="4" t="n"/>
-      <c r="J2191" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2191" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -57612,7 +57612,7 @@
       </c>
       <c r="I2203" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>"No payments found." – Order #2 (CASH, $75.00) için ödeme kaydı listelenmiyor. (Bug: SCRUM-265)</t>
         </is>
       </c>
       <c r="J2203" s="8" t="n"/>
@@ -57712,9 +57712,9 @@
         </is>
       </c>
       <c r="I2206" s="4" t="n"/>
-      <c r="J2206" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2206" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -57905,7 +57905,7 @@
       </c>
       <c r="I2214" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>"No payments found." – Order #2 (CASH, $75.00) için ödeme kaydı listelenmiyor. (Bug: SCRUM-265)</t>
         </is>
       </c>
       <c r="J2214" s="8" t="n"/>
@@ -58004,9 +58004,9 @@
         </is>
       </c>
       <c r="I2217" s="4" t="n"/>
-      <c r="J2217" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2217" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -58193,7 +58193,7 @@
       </c>
       <c r="I2225" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Add. Cat. Management paneli: Mezeler, Soslar, Salata Soslari (Active).</t>
         </is>
       </c>
       <c r="J2225" s="8" t="n"/>
@@ -58292,9 +58292,9 @@
         </is>
       </c>
       <c r="I2228" s="4" t="n"/>
-      <c r="J2228" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2228" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -58481,7 +58481,7 @@
       </c>
       <c r="I2236" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Additions sayfasında 12 ilave ve ek kategorileri listelendi.</t>
         </is>
       </c>
       <c r="J2236" s="8" t="n"/>
@@ -58580,9 +58580,9 @@
         </is>
       </c>
       <c r="I2239" s="4" t="n"/>
-      <c r="J2239" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2239" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -58769,7 +58769,7 @@
       </c>
       <c r="I2247" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>ID, Name, Description, Price, Category kolonları görüntülendi.</t>
         </is>
       </c>
       <c r="J2247" s="8" t="n"/>
@@ -58868,9 +58868,9 @@
         </is>
       </c>
       <c r="I2250" s="4" t="n"/>
-      <c r="J2250" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2250" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -59183,7 +59183,7 @@
       </c>
       <c r="I2263" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>"QA YK Ek" / 3 / Soslar → "Addition added successfully!", listede görüntülendi.</t>
         </is>
       </c>
       <c r="J2263" s="8" t="n"/>
@@ -59282,9 +59282,9 @@
         </is>
       </c>
       <c r="I2266" s="4" t="n"/>
-      <c r="J2266" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2266" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -59593,7 +59593,7 @@
       </c>
       <c r="I2279" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Name boş → kayıt oluştu (adı boş ilave). (Bug: SCRUM-261)</t>
         </is>
       </c>
       <c r="J2279" s="8" t="n"/>
@@ -59692,9 +59692,9 @@
         </is>
       </c>
       <c r="I2282" s="4" t="n"/>
-      <c r="J2282" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2282" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -60003,7 +60003,7 @@
       </c>
       <c r="I2295" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Description boş → kayıt oluştu. (Bug: SCRUM-261)</t>
         </is>
       </c>
       <c r="J2295" s="8" t="n"/>
@@ -60102,9 +60102,9 @@
         </is>
       </c>
       <c r="I2298" s="4" t="n"/>
-      <c r="J2298" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2298" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -60413,7 +60413,7 @@
       </c>
       <c r="I2311" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Price boş → kayıt oluşmadı ancak hiçbir uyarı görüntülenmedi, modal açık kaldı (sessiz hata). (Bug: SCRUM-262)</t>
         </is>
       </c>
       <c r="J2311" s="8" t="n"/>
@@ -60512,9 +60512,9 @@
         </is>
       </c>
       <c r="I2314" s="4" t="n"/>
-      <c r="J2314" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2314" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -60823,7 +60823,7 @@
       </c>
       <c r="I2327" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Addition Category boş → kayıt oluşmadı ancak hiçbir uyarı görüntülenmedi, modal açık kaldı (sessiz hata). (Bug: SCRUM-262)</t>
         </is>
       </c>
       <c r="J2327" s="8" t="n"/>
@@ -60922,9 +60922,9 @@
         </is>
       </c>
       <c r="I2330" s="4" t="n"/>
-      <c r="J2330" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2330" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -61207,7 +61207,7 @@
       </c>
       <c r="I2342" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Sadece Price + Addition Category → kayıt oluşmadı ancak hiçbir uyarı görüntülenmedi (sessiz hata). (Bug: SCRUM-262)</t>
         </is>
       </c>
       <c r="J2342" s="8" t="n"/>
@@ -61307,9 +61307,9 @@
         </is>
       </c>
       <c r="I2345" s="4" t="n"/>
-      <c r="J2345" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2345" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -61522,7 +61522,7 @@
       </c>
       <c r="I2354" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Test ilaveleri silindi → "Addition deleted successfully!", listeden kaldırıldı.</t>
         </is>
       </c>
       <c r="J2354" s="8" t="n"/>
@@ -63544,9 +63544,9 @@
         </is>
       </c>
       <c r="I2431" s="4" t="n"/>
-      <c r="J2431" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2431" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -63771,7 +63771,7 @@
       </c>
       <c r="I2440" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Support Requests'te ID 107 "Yıldıray QA / yk.qa.test@example.com" mesajı görüntülendi.</t>
         </is>
       </c>
       <c r="J2440" s="8" t="n"/>
@@ -63871,9 +63871,9 @@
         </is>
       </c>
       <c r="I2443" s="4" t="n"/>
-      <c r="J2443" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2443" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -64060,7 +64060,7 @@
       </c>
       <c r="I2451" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Support Requests ID, Name, Email, Subject ile listelendi (7 sayfa).</t>
         </is>
       </c>
       <c r="J2451" s="8" t="n"/>
@@ -64160,9 +64160,9 @@
         </is>
       </c>
       <c r="I2454" s="4" t="n"/>
-      <c r="J2454" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2454" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -64371,7 +64371,7 @@
       </c>
       <c r="I2463" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Göz ikonu → Message Details: Name, Email, Subject, Message, Date görüntülendi.</t>
         </is>
       </c>
       <c r="J2463" s="8" t="n"/>
@@ -64471,9 +64471,9 @@
         </is>
       </c>
       <c r="I2466" s="4" t="n"/>
-      <c r="J2466" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2466" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -64686,7 +64686,7 @@
       </c>
       <c r="I2475" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>"All" + Search → tüm mesajlar listelendi.</t>
         </is>
       </c>
       <c r="J2475" s="8" t="n"/>
@@ -64786,9 +64786,9 @@
         </is>
       </c>
       <c r="I2478" s="4" t="n"/>
-      <c r="J2478" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2478" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -65027,7 +65027,7 @@
       </c>
       <c r="I2488" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Email filtresi seçilip "yk.qa.test@example.com" ile aratıldı → liste filtrelenmedi; ayrıca Email kutusu klavye girişini zaman zaman kabul etmiyor. (Bug: SCRUM-263)</t>
         </is>
       </c>
       <c r="J2488" s="8" t="n"/>
@@ -65127,9 +65127,9 @@
         </is>
       </c>
       <c r="I2491" s="4" t="n"/>
-      <c r="J2491" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2491" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -65368,7 +65368,7 @@
       </c>
       <c r="I2501" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Subject = "Schema check" → yalnızca ID 112 listelendi.</t>
         </is>
       </c>
       <c r="J2501" s="8" t="n"/>
@@ -65468,9 +65468,9 @@
         </is>
       </c>
       <c r="I2504" s="4" t="n"/>
-      <c r="J2504" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2504" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -65709,7 +65709,7 @@
       </c>
       <c r="I2514" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Date 10.10.2026–10.10.2026 → mesajlar listelendi; 01.01.2020 → mesaj listelenmedi.</t>
         </is>
       </c>
       <c r="J2514" s="8" t="n"/>
@@ -65809,9 +65809,9 @@
         </is>
       </c>
       <c r="I2517" s="4" t="n"/>
-      <c r="J2517" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2517" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -66050,7 +66050,7 @@
       </c>
       <c r="I2527" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Time 11:00–11:05 → 10:39 ve 10:51 tarihli mesajlar da listelendi; filtre doğru çalışmıyor. (Bug: SCRUM-268)</t>
         </is>
       </c>
       <c r="J2527" s="8" t="n"/>
@@ -66150,9 +66150,9 @@
         </is>
       </c>
       <c r="I2530" s="4" t="n"/>
-      <c r="J2530" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2530" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -66365,7 +66365,7 @@
       </c>
       <c r="I2539" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Eşleşmeyen tarih (01.01.2020) → mesaj listelenmedi ancak bilgilendirme mesajı yok ve sayfalama hâlâ 7 sayfa gösteriyor. (Bug: SCRUM-269)</t>
         </is>
       </c>
       <c r="J2539" s="8" t="n"/>
@@ -66676,7 +66676,7 @@
       </c>
       <c r="I2551" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Admin hesabı gerekli. Test ortamında Admin kullanıcısı paylaşılmadı; Swagger POST /auth/registerAdmin yetki istediği için (401 Unauthorized) Admin hesabı oluşturulamadı. Admin bilgisi eğitmenden talep edildi.</t>
+          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
         </is>
       </c>
       <c r="J2551" s="8" t="n"/>
@@ -68143,13 +68143,13 @@
         <v>2</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K11" s="4" t="n">
         <v>0</v>
@@ -68186,13 +68186,13 @@
         <v>2</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I12" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>0</v>
@@ -68229,13 +68229,13 @@
         <v>1</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K13" s="4" t="n">
         <v>0</v>
@@ -68272,13 +68272,13 @@
         <v>1</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I14" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>0</v>
@@ -68315,13 +68315,13 @@
         <v>7</v>
       </c>
       <c r="H15" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J15" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="I15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="4" t="n">
-        <v>12</v>
       </c>
       <c r="K15" s="4" t="n">
         <v>0</v>
@@ -68358,13 +68358,13 @@
         <v>1</v>
       </c>
       <c r="H16" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="I16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="4" t="n">
-        <v>8</v>
       </c>
       <c r="K16" s="4" t="n">
         <v>0</v>
@@ -68401,13 +68401,13 @@
         <v>1</v>
       </c>
       <c r="H17" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="I17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="K17" s="4" t="n">
         <v>0</v>
@@ -68444,13 +68444,13 @@
         <v>1</v>
       </c>
       <c r="H18" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="I18" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="K18" s="4" t="n">
         <v>0</v>
@@ -68487,13 +68487,13 @@
         <v>0</v>
       </c>
       <c r="H19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J19" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="I19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="K19" s="4" t="n">
         <v>0</v>
@@ -68530,13 +68530,13 @@
         <v>5</v>
       </c>
       <c r="H20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J20" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="I20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="4" t="n">
-        <v>10</v>
       </c>
       <c r="K20" s="4" t="n">
         <v>0</v>
@@ -68573,13 +68573,13 @@
         <v>6</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I21" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J21" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K21" s="4" t="n">
         <v>0</v>
@@ -68616,13 +68616,13 @@
         <v>1</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="K22" s="4" t="n">
         <v>0</v>
@@ -68647,13 +68647,13 @@
         <v>91</v>
       </c>
       <c r="H23" s="12" t="n">
-        <v>53</v>
+        <v>99</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="J23" s="12" t="n">
-        <v>107</v>
+        <v>43</v>
       </c>
       <c r="K23" s="12" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Manuel koşum tamamlandı: 192 test case (128 PASSED / 64 FAILED); SCRUM-270..272
Kalan admin kayıt/giriş, silme ve sipariş statüsü test case'leri koşuldu.
Test case dosyası, Test Planı v1.2 ve Xray execution sonuç dosyası güncellendi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Snack_Attack_Test_Cases_Yildiray_Kosedag.xlsx
+++ b/docs/Snack_Attack_Test_Cases_Yildiray_Kosedag.xlsx
@@ -47,7 +47,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -72,11 +72,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0038761D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E69138"/>
       </patternFill>
     </fill>
   </fills>
@@ -139,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -163,9 +158,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -7970,7 +7962,11 @@
         </is>
       </c>
       <c r="I291" s="4" t="n"/>
-      <c r="J291" s="2" t="n"/>
+      <c r="J291" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="7" t="n"/>
@@ -8291,7 +8287,11 @@
           <t>Email'in zaten kayıtlı olduğuna dair uyarı mesajı görüntülenmeli, kayıt yapılmamalıdır</t>
         </is>
       </c>
-      <c r="I304" s="4" t="n"/>
+      <c r="I304" s="4" t="inlineStr">
+        <is>
+          <t>Kayıtlı email (kosedagyildiray5@gmail.com) ile Register → "Error : User with email kosedagyildiray5@gmail.com is ALREADY REGISTERED", kayıt yapılmadı.</t>
+        </is>
+      </c>
       <c r="J304" s="8" t="n"/>
     </row>
     <row r="305">
@@ -10092,7 +10092,11 @@
         </is>
       </c>
       <c r="I370" s="4" t="n"/>
-      <c r="J370" s="2" t="n"/>
+      <c r="J370" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="7" t="n"/>
@@ -10209,7 +10213,11 @@
           <t>Giriş yapılmamalı; login sayfasında anlaşılır bir hata mesajı (ör. "Sign in failed. Check the details you provided are correct.") görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I375" s="4" t="n"/>
+      <c r="I375" s="4" t="inlineStr">
+        <is>
+          <t>Kayıtlı email + yanlış şifre → giriş yapılmadı ancak ham "CredentialsSignin" görüntülendi. (Bug: SCRUM-271)</t>
+        </is>
+      </c>
       <c r="J375" s="8" t="n"/>
     </row>
     <row r="377">
@@ -10305,7 +10313,11 @@
         </is>
       </c>
       <c r="I378" s="4" t="n"/>
-      <c r="J378" s="2" t="n"/>
+      <c r="J378" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="7" t="n"/>
@@ -10422,7 +10434,11 @@
           <t>Giriş yapılmamalı; login sayfasında anlaşılır bir hata mesajı görüntülenmelidir</t>
         </is>
       </c>
-      <c r="I383" s="4" t="n"/>
+      <c r="I383" s="4" t="inlineStr">
+        <is>
+          <t>Kayıtsız email → giriş yapılmadı ancak ham "CredentialsSignin" görüntülendi. (Bug: SCRUM-271)</t>
+        </is>
+      </c>
       <c r="J383" s="8" t="n"/>
     </row>
     <row r="385">
@@ -10915,9 +10931,9 @@
         </is>
       </c>
       <c r="I400" s="4" t="n"/>
-      <c r="J400" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J400" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -11360,7 +11376,7 @@
       </c>
       <c r="I418" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Geçerli verilerle kayıt başarılı (Admin Management'ta ID 20 "QA YKAdmin" listelendi) ancak "Success" yerine "Registration successful! You can now log in." mesajı görüntülendi. (Bug: SCRUM-270)</t>
         </is>
       </c>
       <c r="J418" s="8" t="n"/>
@@ -11467,9 +11483,9 @@
         </is>
       </c>
       <c r="I422" s="4" t="n"/>
-      <c r="J422" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J422" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -11908,7 +11924,7 @@
       </c>
       <c r="I440" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Admin Management &gt; New formunda FirstName boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J440" s="8" t="n"/>
@@ -12015,9 +12031,9 @@
         </is>
       </c>
       <c r="I444" s="4" t="n"/>
-      <c r="J444" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J444" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -12456,7 +12472,7 @@
       </c>
       <c r="I462" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Admin Management &gt; New formunda LastName boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J462" s="8" t="n"/>
@@ -12563,9 +12579,9 @@
         </is>
       </c>
       <c r="I466" s="4" t="n"/>
-      <c r="J466" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J466" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -13004,7 +13020,7 @@
       </c>
       <c r="I484" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Admin Management &gt; New formunda Phone Number boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J484" s="8" t="n"/>
@@ -13111,9 +13127,9 @@
         </is>
       </c>
       <c r="I488" s="4" t="n"/>
-      <c r="J488" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J488" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -13552,7 +13568,7 @@
       </c>
       <c r="I506" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Admin Management &gt; New formunda Email boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J506" s="8" t="n"/>
@@ -13659,9 +13675,9 @@
         </is>
       </c>
       <c r="I510" s="4" t="n"/>
-      <c r="J510" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J510" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -14100,7 +14116,7 @@
       </c>
       <c r="I528" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Admin Management &gt; New formunda Username boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J528" s="8" t="n"/>
@@ -14207,9 +14223,9 @@
         </is>
       </c>
       <c r="I532" s="4" t="n"/>
-      <c r="J532" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J532" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -14648,7 +14664,7 @@
       </c>
       <c r="I550" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Admin Management &gt; New formunda Password boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J550" s="8" t="n"/>
@@ -14755,9 +14771,9 @@
         </is>
       </c>
       <c r="I554" s="4" t="n"/>
-      <c r="J554" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J554" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -15196,7 +15212,7 @@
       </c>
       <c r="I572" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Admin Management &gt; New formunda Confirm Password boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J572" s="8" t="n"/>
@@ -15303,9 +15319,9 @@
         </is>
       </c>
       <c r="I576" s="4" t="n"/>
-      <c r="J576" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J576" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -15748,7 +15764,7 @@
       </c>
       <c r="I594" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Password ≠ Confirm Password → "Passwords must match." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J594" s="8" t="n"/>
@@ -15855,9 +15871,9 @@
         </is>
       </c>
       <c r="I598" s="4" t="n"/>
-      <c r="J598" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J598" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -16300,7 +16316,7 @@
       </c>
       <c r="I616" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>+90 (TR) ile Phone "54a1234567" → "Invalid phone number." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J616" s="8" t="n"/>
@@ -16407,9 +16423,9 @@
         </is>
       </c>
       <c r="I620" s="4" t="n"/>
-      <c r="J620" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J620" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -16852,7 +16868,7 @@
       </c>
       <c r="I638" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>+90 (TR) ile Phone "541-123-45!" → "Invalid phone number." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J638" s="8" t="n"/>
@@ -16959,9 +16975,9 @@
         </is>
       </c>
       <c r="I642" s="4" t="n"/>
-      <c r="J642" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J642" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -17404,7 +17420,7 @@
       </c>
       <c r="I660" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>+90 (TR) ile Phone "54112345 (8 hane)" → "Invalid phone number." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J660" s="8" t="n"/>
@@ -17511,9 +17527,9 @@
         </is>
       </c>
       <c r="I664" s="4" t="n"/>
-      <c r="J664" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J664" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -17956,7 +17972,7 @@
       </c>
       <c r="I682" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>+90 (TR) ile Phone "541123456789 (12 hane)" → "Invalid phone number." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J682" s="8" t="n"/>
@@ -18063,9 +18079,9 @@
         </is>
       </c>
       <c r="I686" s="4" t="n"/>
-      <c r="J686" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J686" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -18508,7 +18524,7 @@
       </c>
       <c r="I704" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>+1 (US) seçili, Phone "5411234567" (TR numarası) → "Invalid phone number." görüntülendi.</t>
         </is>
       </c>
       <c r="J704" s="8" t="n"/>
@@ -18615,9 +18631,9 @@
         </is>
       </c>
       <c r="I708" s="4" t="n"/>
-      <c r="J708" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J708" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -19056,7 +19072,7 @@
       </c>
       <c r="I726" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Admin Management &gt; New formunda Region Code boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J726" s="8" t="n"/>
@@ -19163,9 +19179,9 @@
         </is>
       </c>
       <c r="I730" s="4" t="n"/>
-      <c r="J730" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J730" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -19604,7 +19620,7 @@
       </c>
       <c r="I748" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Admin Management &gt; New formunda Address boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J748" s="8" t="n"/>
@@ -19711,9 +19727,9 @@
         </is>
       </c>
       <c r="I752" s="4" t="n"/>
-      <c r="J752" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J752" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -20156,7 +20172,7 @@
       </c>
       <c r="I770" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Email "alican" → "Invalid email address." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J770" s="8" t="n"/>
@@ -20262,9 +20278,9 @@
         </is>
       </c>
       <c r="I774" s="4" t="n"/>
-      <c r="J774" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J774" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -20707,7 +20723,7 @@
       </c>
       <c r="I792" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Kayıtlı email (mehmet@admin.com) → "Error : User with email mehmet@admin.com is ALREADY REGISTERED", kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J792" s="8" t="n"/>
@@ -20814,9 +20830,9 @@
         </is>
       </c>
       <c r="I796" s="4" t="n"/>
-      <c r="J796" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J796" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -21033,7 +21049,7 @@
       </c>
       <c r="I805" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Password ve Confirm Password alanları type="password"; girilen değer maskelenmiş (●●●) görüntülendi.</t>
         </is>
       </c>
       <c r="J805" s="8" t="n"/>
@@ -21132,9 +21148,9 @@
         </is>
       </c>
       <c r="I808" s="4" t="n"/>
-      <c r="J808" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J808" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -21277,7 +21293,7 @@
       </c>
       <c r="I814" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>mehmet@admin.com ile "Login successful!"; /dashboard/admin "Welcome to Admin Panel" ve yönetim menüleri görüntülendi.</t>
         </is>
       </c>
       <c r="J814" s="8" t="n"/>
@@ -21383,9 +21399,9 @@
         </is>
       </c>
       <c r="I818" s="4" t="n"/>
-      <c r="J818" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J818" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -21506,7 +21522,7 @@
       </c>
       <c r="I823" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Email "mehmetadmin.com" → "Invalid email" yerine "Invalid email address" görüntülendi. (Bug: SCRUM-33)</t>
         </is>
       </c>
       <c r="J823" s="8" t="n"/>
@@ -21605,9 +21621,9 @@
         </is>
       </c>
       <c r="I826" s="4" t="n"/>
-      <c r="J826" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J826" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -21728,7 +21744,7 @@
       </c>
       <c r="I831" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Email "mehmet@admincom" için hiçbir uyarı görüntülenmedi. (Bug: SCRUM-236)</t>
         </is>
       </c>
       <c r="J831" s="8" t="n"/>
@@ -21827,9 +21843,9 @@
         </is>
       </c>
       <c r="I834" s="4" t="n"/>
-      <c r="J834" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J834" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -21946,7 +21962,7 @@
       </c>
       <c r="I839" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Password boşken "Password is required" yerine "Required" görüntülendi. (Bug: SCRUM-32)</t>
         </is>
       </c>
       <c r="J839" s="8" t="n"/>
@@ -22045,9 +22061,9 @@
         </is>
       </c>
       <c r="I842" s="4" t="n"/>
-      <c r="J842" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J842" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -22138,7 +22154,7 @@
       </c>
       <c r="I846" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Email ve Password boşken Login butonu aktif (disabled=false); tıklanınca "Required" uyarıları çıkıyor. (Bug: SCRUM-31)</t>
         </is>
       </c>
       <c r="J846" s="8" t="n"/>
@@ -22237,9 +22253,9 @@
         </is>
       </c>
       <c r="I849" s="4" t="n"/>
-      <c r="J849" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J849" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -22334,7 +22350,7 @@
       </c>
       <c r="I853" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Yalnızca Email girili iken Login butonu aktif. (Bug: SCRUM-31)</t>
         </is>
       </c>
       <c r="J853" s="8" t="n"/>
@@ -22433,9 +22449,9 @@
         </is>
       </c>
       <c r="I856" s="4" t="n"/>
-      <c r="J856" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J856" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -22530,7 +22546,7 @@
       </c>
       <c r="I860" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Yalnızca Password girili iken Login butonu aktif. (Bug: SCRUM-31)</t>
         </is>
       </c>
       <c r="J860" s="8" t="n"/>
@@ -22629,9 +22645,9 @@
         </is>
       </c>
       <c r="I863" s="4" t="n"/>
-      <c r="J863" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J863" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -22752,7 +22768,7 @@
       </c>
       <c r="I868" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Kayıtlı email + yanlış şifre → giriş yapılmadı ancak anlaşılır mesaj yerine ham "CredentialsSignin" görüntülendi. (Bug: SCRUM-271)</t>
         </is>
       </c>
       <c r="J868" s="8" t="n"/>
@@ -22850,9 +22866,9 @@
         </is>
       </c>
       <c r="I871" s="4" t="n"/>
-      <c r="J871" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J871" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -22973,7 +22989,7 @@
       </c>
       <c r="I876" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Kayıtsız email → giriş yapılmadı ancak ham "CredentialsSignin" görüntülendi. (Bug: SCRUM-271)</t>
         </is>
       </c>
       <c r="J876" s="8" t="n"/>
@@ -23071,9 +23087,9 @@
         </is>
       </c>
       <c r="I879" s="4" t="n"/>
-      <c r="J879" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J879" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -23146,7 +23162,7 @@
       </c>
       <c r="I882" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Şifre girişi gerektiriyor; kullanıcı tarafından manuel koşulacak.</t>
+          <t>Password alanı type="password"; girilen şifre maskelenmiş görüntülendi.</t>
         </is>
       </c>
       <c r="J882" s="8" t="n"/>
@@ -35086,9 +35102,9 @@
         </is>
       </c>
       <c r="I1331" s="4" t="n"/>
-      <c r="J1331" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1331" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -35253,7 +35269,7 @@
       </c>
       <c r="I1338" s="4" t="inlineStr">
         <is>
-          <t>Bloke – CONFIRMED/DELIVERED durumunda sipariş için Admin/Seller hesabı gerekli.</t>
+          <t>CONFIRMED siparişte Cancel Order butonu görünür ve aktif; onaylanınca "Failed to cancel the order." (iptal olmadı ama buton gizlenmiyor/pasif değil). (Bug: SCRUM-254)</t>
         </is>
       </c>
       <c r="J1338" s="8" t="n"/>
@@ -35353,9 +35369,9 @@
         </is>
       </c>
       <c r="I1341" s="4" t="n"/>
-      <c r="J1341" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1341" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -35520,7 +35536,7 @@
       </c>
       <c r="I1348" s="4" t="inlineStr">
         <is>
-          <t>Bloke – CONFIRMED/DELIVERED durumunda sipariş için Admin/Seller hesabı gerekli.</t>
+          <t>DELIVERED siparişte Cancel Order butonu görünür ve aktif; onaylanınca "Failed to cancel the order.". (Bug: SCRUM-254)</t>
         </is>
       </c>
       <c r="J1348" s="8" t="n"/>
@@ -36495,9 +36511,9 @@
         </is>
       </c>
       <c r="I1384" s="4" t="n"/>
-      <c r="J1384" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1384" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -36688,7 +36704,7 @@
       </c>
       <c r="I1392" s="4" t="inlineStr">
         <is>
-          <t>Bloke – CONFIRMED durumunda sipariş oluşturmak için Admin/Seller hesabı gerekli. Ayrıca sayfada durum filtresi yok (SCRUM-253). (Bug: SCRUM-253)</t>
+          <t>CONFIRMED Order #2 listelendi ancak statü filtresi yok, "CONFIRMED" seçilemiyor. (Bug: SCRUM-253)</t>
         </is>
       </c>
       <c r="J1392" s="8" t="n"/>
@@ -36788,9 +36804,9 @@
         </is>
       </c>
       <c r="I1395" s="4" t="n"/>
-      <c r="J1395" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1395" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -36981,7 +36997,7 @@
       </c>
       <c r="I1403" s="4" t="inlineStr">
         <is>
-          <t>Bloke – DELIVERED durumunda sipariş oluşturmak için Admin/Seller hesabı gerekli. Ayrıca sayfada durum filtresi yok (SCRUM-253). (Bug: SCRUM-253)</t>
+          <t>DELIVERED Order #2 listelendi ancak statü filtresi yok, "DELIVERED" seçilemiyor. (Bug: SCRUM-253)</t>
         </is>
       </c>
       <c r="J1403" s="8" t="n"/>
@@ -37983,9 +37999,9 @@
         </is>
       </c>
       <c r="I1441" s="4" t="n"/>
-      <c r="J1441" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1441" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -38220,7 +38236,7 @@
       </c>
       <c r="I1451" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
+          <t>Test kullanıcısı (ID 21, kosedagyildiray5+qa1@gmail.com) silindi, listeden kaldırıldı. Not: başarı mesajı görüntülenmedi.</t>
         </is>
       </c>
       <c r="J1451" s="8" t="n"/>
@@ -38319,9 +38335,9 @@
         </is>
       </c>
       <c r="I1454" s="4" t="n"/>
-      <c r="J1454" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1454" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -38534,7 +38550,7 @@
       </c>
       <c r="I1463" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
+          <t>Silme onayında İptal → kullanıcı listede kaldı. Not: onay metni "delete this admin?" (yanlış metin).</t>
         </is>
       </c>
       <c r="J1463" s="8" t="n"/>
@@ -38634,9 +38650,9 @@
         </is>
       </c>
       <c r="I1466" s="4" t="n"/>
-      <c r="J1466" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1466" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -38709,7 +38725,7 @@
       </c>
       <c r="I1469" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
+          <t>Silinen kullanıcı ile giriş yapılamadı ("CredentialsSignin"). Not: aktivasyon maili gelmediğinden hesap silme öncesinde de aktif değildi.</t>
         </is>
       </c>
       <c r="J1469" s="8" t="n"/>
@@ -39437,9 +39453,9 @@
         </is>
       </c>
       <c r="I1496" s="4" t="n"/>
-      <c r="J1496" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1496" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -39674,7 +39690,7 @@
       </c>
       <c r="I1506" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
+          <t>Test admini (ID 20, qa.ykadmin1@example.com) silindi, listeden kaldırıldı. Not: başarı mesajı görüntülenmedi.</t>
         </is>
       </c>
       <c r="J1506" s="8" t="n"/>
@@ -39773,9 +39789,9 @@
         </is>
       </c>
       <c r="I1509" s="4" t="n"/>
-      <c r="J1509" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1509" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -39988,7 +40004,7 @@
       </c>
       <c r="I1518" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
+          <t>"Are you sure you want to delete this admin?" onayında İptal → admin listede kaldı.</t>
         </is>
       </c>
       <c r="J1518" s="8" t="n"/>
@@ -40087,9 +40103,9 @@
         </is>
       </c>
       <c r="I1521" s="4" t="n"/>
-      <c r="J1521" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1521" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -40302,7 +40318,7 @@
       </c>
       <c r="I1530" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
+          <t>admin@example.com satırında Delete butonu aktif; uyarı olmadan silme onayı soruluyor (onay İptal edildi, hesap silinmedi). (Bug: SCRUM-272)</t>
         </is>
       </c>
       <c r="J1530" s="8" t="n"/>
@@ -41310,9 +41326,9 @@
         </is>
       </c>
       <c r="I1568" s="4" t="n"/>
-      <c r="J1568" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1568" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -41547,7 +41563,7 @@
       </c>
       <c r="I1578" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
+          <t>Order #2 CONFIRMED yapıldı → "Order status updated."; kullanıcı My Orders'ta "Status: CONFIRMED". Not: PENDING sipariş olmadığından admin panelinde PENDING görünen Order #2 kullanıldı.</t>
         </is>
       </c>
       <c r="J1578" s="8" t="n"/>
@@ -41647,9 +41663,9 @@
         </is>
       </c>
       <c r="I1581" s="4" t="n"/>
-      <c r="J1581" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1581" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -41884,7 +41900,7 @@
       </c>
       <c r="I1591" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
+          <t>Order #2 DELIVERED yapıldı → "Order status updated."; kullanıcı My Orders'ta "Status: DELIVERED".</t>
         </is>
       </c>
       <c r="J1591" s="8" t="n"/>
@@ -41984,9 +42000,9 @@
         </is>
       </c>
       <c r="I1594" s="4" t="n"/>
-      <c r="J1594" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J1594" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -42199,7 +42215,7 @@
       </c>
       <c r="I1603" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak. Not: CANCELED Order #2'nin statü dropdown'ı aktif görünüyor. (Bug: SCRUM-264)</t>
+          <t>CANCELED Order #2'nin statüsü CONFIRMED yapılabildi ("Order status updated."); pasif/uyarı yok. (Bug: SCRUM-264)</t>
         </is>
       </c>
       <c r="J1603" s="8" t="n"/>
@@ -66465,9 +66481,9 @@
         </is>
       </c>
       <c r="I2542" s="4" t="n"/>
-      <c r="J2542" s="11" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J2542" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -66676,7 +66692,7 @@
       </c>
       <c r="I2551" s="4" t="inlineStr">
         <is>
-          <t>Bloke – Ortak test ortamında veri değiştiren bu adım (hesap oluşturma/silme, sipariş statüsü değiştirme veya mesaj silme) kullanıcı tarafından koşulacak.</t>
+          <t>Test mesajı (ID 115) silindi → "Message deleted successfully", listeden kaldırıldı.</t>
         </is>
       </c>
       <c r="J2551" s="8" t="n"/>
@@ -67756,7 +67772,7 @@
         <v>17</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I2" s="4" t="n">
         <v>2</v>
@@ -67765,7 +67781,7 @@
         <v>0</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -67802,13 +67818,13 @@
         <v>2</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J3" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -67842,13 +67858,13 @@
         <v>17</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>19</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>0</v>
@@ -67885,13 +67901,13 @@
         <v>8</v>
       </c>
       <c r="H5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="J5" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="4" t="n">
-        <v>10</v>
       </c>
       <c r="K5" s="4" t="n">
         <v>0</v>
@@ -68060,10 +68076,10 @@
         <v>6</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K9" s="4" t="n">
         <v>0</v>
@@ -68103,10 +68119,10 @@
         <v>1</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>0</v>
@@ -68143,13 +68159,13 @@
         <v>2</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K11" s="4" t="n">
         <v>0</v>
@@ -68186,13 +68202,13 @@
         <v>2</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>3</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>0</v>
@@ -68229,13 +68245,13 @@
         <v>1</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K13" s="4" t="n">
         <v>0</v>
@@ -68616,99 +68632,99 @@
         <v>1</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I22" s="4" t="n">
         <v>3</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K22" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>TOPLAM</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr"/>
-      <c r="C23" s="12" t="inlineStr"/>
-      <c r="D23" s="12" t="inlineStr"/>
-      <c r="E23" s="12" t="n">
+      <c r="B23" s="11" t="inlineStr"/>
+      <c r="C23" s="11" t="inlineStr"/>
+      <c r="D23" s="11" t="inlineStr"/>
+      <c r="E23" s="11" t="n">
         <v>192</v>
       </c>
-      <c r="F23" s="12" t="n">
+      <c r="F23" s="11" t="n">
         <v>101</v>
       </c>
-      <c r="G23" s="12" t="n">
+      <c r="G23" s="11" t="n">
         <v>91</v>
       </c>
-      <c r="H23" s="12" t="n">
-        <v>99</v>
-      </c>
-      <c r="I23" s="12" t="n">
-        <v>47</v>
-      </c>
-      <c r="J23" s="12" t="n">
-        <v>43</v>
-      </c>
-      <c r="K23" s="12" t="n">
-        <v>3</v>
+      <c r="H23" s="11" t="n">
+        <v>128</v>
+      </c>
+      <c r="I23" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="J23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>Test Datası Yer Tutucuları</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="14" t="inlineStr">
+      <c r="A26" s="13" t="inlineStr">
         <is>
           <t>{Email} / {Username} / {PhoneNumber}</t>
         </is>
       </c>
-      <c r="B26" s="14" t="inlineStr">
+      <c r="B26" s="13" t="inlineStr">
         <is>
           <t>Her koşumda benzersiz üretilen kayıt dataları</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="14" t="inlineStr">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>{UserEmail} / {UserPassword}</t>
         </is>
       </c>
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Aktif User test hesabı (configuration dosyasında saklanır)</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="14" t="inlineStr">
+      <c r="A28" s="13" t="inlineStr">
         <is>
           <t>{AdminEmail} / {AdminPassword}</t>
         </is>
       </c>
-      <c r="B28" s="14" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>Aktif Admin test hesabı (eğitmenden / registerAdmin ile)</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="inlineStr">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>{Unique}</t>
         </is>
       </c>
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Zaman damgası ile benzersiz değer</t>
         </is>

</xml_diff>

<commit_message>
Test sonuçları beklenen sonuçlara göre denetlendi: 120 PASSED / 72 FAILED; SCRUM-273..275
Beklenen başarı/bilgilendirme mesajı veya bilgi alanı bulunmayan 8 test case
FAILED olarak düzeltildi; US_13 TC_02 kategori filtresi koşuldu; US_03 sonuç
metinleri gerçekte yapılan adımlara göre düzeltildi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Snack_Attack_Test_Cases_Yildiray_Kosedag.xlsx
+++ b/docs/Snack_Attack_Test_Cases_Yildiray_Kosedag.xlsx
@@ -11924,7 +11924,7 @@
       </c>
       <c r="I440" s="4" t="inlineStr">
         <is>
-          <t>Admin Management &gt; New formunda FirstName boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
+          <t>Admin Management &gt; New formu boş gönderildiğinde (Register) FirstName alanının altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J440" s="8" t="n"/>
@@ -12472,7 +12472,7 @@
       </c>
       <c r="I462" s="4" t="inlineStr">
         <is>
-          <t>Admin Management &gt; New formunda LastName boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
+          <t>Admin Management &gt; New formu boş gönderildiğinde (Register) LastName alanının altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J462" s="8" t="n"/>
@@ -13020,7 +13020,7 @@
       </c>
       <c r="I484" s="4" t="inlineStr">
         <is>
-          <t>Admin Management &gt; New formunda Phone Number boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
+          <t>Admin Management &gt; New formu boş gönderildiğinde (Register) Phone Number alanının altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J484" s="8" t="n"/>
@@ -13568,7 +13568,7 @@
       </c>
       <c r="I506" s="4" t="inlineStr">
         <is>
-          <t>Admin Management &gt; New formunda Email boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
+          <t>Admin Management &gt; New formu boş gönderildiğinde (Register) Email alanının altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J506" s="8" t="n"/>
@@ -14116,7 +14116,7 @@
       </c>
       <c r="I528" s="4" t="inlineStr">
         <is>
-          <t>Admin Management &gt; New formunda Username boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
+          <t>Admin Management &gt; New formu boş gönderildiğinde (Register) Username alanının altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J528" s="8" t="n"/>
@@ -14664,7 +14664,7 @@
       </c>
       <c r="I550" s="4" t="inlineStr">
         <is>
-          <t>Admin Management &gt; New formunda Password boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
+          <t>Admin Management &gt; New formu boş gönderildiğinde (Register) Password alanının altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J550" s="8" t="n"/>
@@ -15212,7 +15212,7 @@
       </c>
       <c r="I572" s="4" t="inlineStr">
         <is>
-          <t>Admin Management &gt; New formunda Confirm Password boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
+          <t>Admin Management &gt; New formu boş gönderildiğinde (Register) Confirm Password alanının altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J572" s="8" t="n"/>
@@ -19072,7 +19072,7 @@
       </c>
       <c r="I726" s="4" t="inlineStr">
         <is>
-          <t>Admin Management &gt; New formunda Region Code boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
+          <t>Admin Management &gt; New formu boş gönderildiğinde (Register) Region Code alanının altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J726" s="8" t="n"/>
@@ -19620,7 +19620,7 @@
       </c>
       <c r="I748" s="4" t="inlineStr">
         <is>
-          <t>Admin Management &gt; New formunda Address boşken Register → alanın altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
+          <t>Admin Management &gt; New formu boş gönderildiğinde (Register) Address alanının altında "This field is required." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J748" s="8" t="n"/>
@@ -37999,9 +37999,9 @@
         </is>
       </c>
       <c r="I1441" s="4" t="n"/>
-      <c r="J1441" s="10" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+      <c r="J1441" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -38236,7 +38236,7 @@
       </c>
       <c r="I1451" s="4" t="inlineStr">
         <is>
-          <t>Test kullanıcısı (ID 21, kosedagyildiray5+qa1@gmail.com) silindi, listeden kaldırıldı. Not: başarı mesajı görüntülenmedi.</t>
+          <t>Test kullanıcısı (ID 21, kosedagyildiray5+qa1@gmail.com) silindi ve listeden kaldırıldı; ancak başarı mesajı görüntülenmedi. (Bug: SCRUM-273)</t>
         </is>
       </c>
       <c r="J1451" s="8" t="n"/>
@@ -39453,9 +39453,9 @@
         </is>
       </c>
       <c r="I1496" s="4" t="n"/>
-      <c r="J1496" s="10" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+      <c r="J1496" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -39690,7 +39690,7 @@
       </c>
       <c r="I1506" s="4" t="inlineStr">
         <is>
-          <t>Test admini (ID 20, qa.ykadmin1@example.com) silindi, listeden kaldırıldı. Not: başarı mesajı görüntülenmedi.</t>
+          <t>Test admini (ID 20, qa.ykadmin1@example.com) silindi ve listeden kaldırıldı; ancak başarı mesajı görüntülenmedi. (Bug: SCRUM-273)</t>
         </is>
       </c>
       <c r="J1506" s="8" t="n"/>
@@ -42314,9 +42314,9 @@
         </is>
       </c>
       <c r="I1606" s="4" t="n"/>
-      <c r="J1606" s="10" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+      <c r="J1606" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -42503,7 +42503,7 @@
       </c>
       <c r="I1614" s="4" t="inlineStr">
         <is>
-          <t>Product Management'ta ürünler ID, Image, Name, Description, Price, Order Count, Category, Created At ile görüntülendi (3 sayfa).</t>
+          <t>Ürünler ID, Image, Name, Description, Price, Order Count, Category, Created At ile görüntülendi; ancak indirim ve Available/Active durumu listede yok. (Bug: SCRUM-274)</t>
         </is>
       </c>
       <c r="J1614" s="8" t="n"/>
@@ -42817,7 +42817,7 @@
       </c>
       <c r="I1626" s="4" t="inlineStr">
         <is>
-          <t>Ürünler sayfalama ile listelendi. Not: tüm ürünlerde Order Count = 35.</t>
+          <t>Admin Product Management'ta "Pizza" filtresi seçildi → yalnızca PIZZA kategorisindeki 6 ürün listelendi.</t>
         </is>
       </c>
       <c r="J1626" s="8" t="n"/>
@@ -43230,9 +43230,9 @@
         </is>
       </c>
       <c r="I1641" s="4" t="n"/>
-      <c r="J1641" s="10" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+      <c r="J1641" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -43445,7 +43445,7 @@
       </c>
       <c r="I1650" s="4" t="inlineStr">
         <is>
-          <t>"zzqxyokurun" araması → ürün listelenmedi. Not: bilgilendirme mesajı yok.</t>
+          <t>"zzqxyokurun" araması → ürün listelenmedi ancak bilgilendirme mesajı görüntülenmedi. (Bug: SCRUM-275)</t>
         </is>
       </c>
       <c r="J1650" s="8" t="n"/>
@@ -44007,7 +44007,7 @@
       </c>
       <c r="I1672" s="4" t="inlineStr">
         <is>
-          <t>"QA YK Tam Urun" (100, indirim 10, HAMBURGER, Soslar, resim) → "Ürün başarıyla oluşturuldu!"; listede ve kullanıcı Products sayfasında görüntülendi. Not: indirim fiyata yansımıyor.</t>
+          <t>"QA YK Tam Urun" (100, indirim 10, HAMBURGER, Soslar, resim) → "Ürün başarıyla oluşturuldu!"; listede ve kullanıcı Products sayfasında görüntülendi. Not: indirim fiyata yansımıyor (SCRUM-259).</t>
         </is>
       </c>
       <c r="J1672" s="8" t="n"/>
@@ -51613,7 +51613,7 @@
       </c>
       <c r="I1971" s="4" t="inlineStr">
         <is>
-          <t>Fiyat 120 ve indirim 20 kaydedildi. Not: indirim kullanıcı tarafında fiyata yansımıyor.</t>
+          <t>Fiyat 100→120 ve indirim 10→20 kaydedildi, düzenleme formunda ve listede yeni fiyat görüntülendi. Not: indirim kullanıcı tarafında fiyata yansımıyor (SCRUM-259); güncelleme sonrası başarı mesajı "Ürün başarıyla güncellendi!".</t>
         </is>
       </c>
       <c r="J1971" s="8" t="n"/>
@@ -54875,9 +54875,9 @@
         </is>
       </c>
       <c r="I2096" s="4" t="n"/>
-      <c r="J2096" s="10" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+      <c r="J2096" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -55064,7 +55064,7 @@
       </c>
       <c r="I2104" s="4" t="inlineStr">
         <is>
-          <t>Category Management Panel: ID, Name, Active, Created At ile 6 kategori görüntülendi.</t>
+          <t>Category Management Panel ID, Name, Active, Created At ile görüntülendi; ancak kategori açıklaması listede yok. (Bug: SCRUM-274)</t>
         </is>
       </c>
       <c r="J2104" s="8" t="n"/>
@@ -55451,9 +55451,9 @@
         </is>
       </c>
       <c r="I2118" s="4" t="n"/>
-      <c r="J2118" s="10" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+      <c r="J2118" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -55714,7 +55714,7 @@
       </c>
       <c r="I2129" s="4" t="inlineStr">
         <is>
-          <t>"QAYKTEST" eklendi, listede görüntülendi (ID 7). Not: başarı mesajı görüntülenmedi.</t>
+          <t>"QAYKTEST" kategorisi eklendi ve listede görüntülendi (ID 7); ancak başarı mesajı görüntülenmedi. (Bug: SCRUM-273)</t>
         </is>
       </c>
       <c r="J2129" s="8" t="n"/>
@@ -56124,9 +56124,9 @@
         </is>
       </c>
       <c r="I2144" s="4" t="n"/>
-      <c r="J2144" s="10" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+      <c r="J2144" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -56339,7 +56339,7 @@
       </c>
       <c r="I2153" s="4" t="inlineStr">
         <is>
-          <t>"QAYKTEST" silindi, listeden kaldırıldı. Not: onay metni "delete this product?" (yanlış metin).</t>
+          <t>"QAYKTEST" silindi ve listeden kaldırıldı; ancak başarı mesajı görüntülenmedi, onay metni "delete this product?" (yanlış metin). (Bug: SCRUM-273)</t>
         </is>
       </c>
       <c r="J2153" s="8" t="n"/>
@@ -63887,9 +63887,9 @@
         </is>
       </c>
       <c r="I2443" s="4" t="n"/>
-      <c r="J2443" s="10" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+      <c r="J2443" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>
@@ -64076,7 +64076,7 @@
       </c>
       <c r="I2451" s="4" t="inlineStr">
         <is>
-          <t>Support Requests ID, Name, Email, Subject ile listelendi (7 sayfa).</t>
+          <t>Support Requests ID, Name, Email, Subject ile listelendi (7 sayfa); ancak Date bilgisi listede yok, yalnızca detay penceresinde görülebiliyor. (Bug: SCRUM-274)</t>
         </is>
       </c>
       <c r="J2451" s="8" t="n"/>
@@ -68159,10 +68159,10 @@
         <v>2</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11" s="4" t="n">
         <v>0</v>
@@ -68202,10 +68202,10 @@
         <v>2</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>0</v>
@@ -68288,10 +68288,10 @@
         <v>1</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>0</v>
@@ -68460,10 +68460,10 @@
         <v>1</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J18" s="4" t="n">
         <v>0</v>
@@ -68632,10 +68632,10 @@
         <v>1</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J22" s="4" t="n">
         <v>0</v>
@@ -68663,10 +68663,10 @@
         <v>91</v>
       </c>
       <c r="H23" s="11" t="n">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="J23" s="11" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Sonuç metinleri düzeltildi: '+' ile başlayan metinler Google Sheets'te formül hatası veriyordu
US_01 TC_14 ve US_03 TC_10-14 sonuç metinleri 'Country Code ...' ile başlayacak
şekilde düzenlendi; Excel ve Xray sonuç dosyası güncellendi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Snack_Attack_Test_Cases_Yildiray_Kosedag.xlsx
+++ b/docs/Snack_Attack_Test_Cases_Yildiray_Kosedag.xlsx
@@ -6565,7 +6565,7 @@
       </c>
       <c r="I236" s="4" t="inlineStr">
         <is>
-          <t>+1 (US) seçili ve TR numarası girili iken "Invalid phone number." uyarısı görüntülendi.</t>
+          <t>Country Code +1 (US) seçili ve TR numarası girili iken "Invalid phone number." uyarısı görüntülendi.</t>
         </is>
       </c>
       <c r="J236" s="8" t="n"/>
@@ -16316,7 +16316,7 @@
       </c>
       <c r="I616" s="4" t="inlineStr">
         <is>
-          <t>+90 (TR) ile Phone "54a1234567" → "Invalid phone number." görüntülendi, kayıt yapılmadı.</t>
+          <t>Country Code +90 (TR), Phone "54a1234567" → "Invalid phone number." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J616" s="8" t="n"/>
@@ -16868,7 +16868,7 @@
       </c>
       <c r="I638" s="4" t="inlineStr">
         <is>
-          <t>+90 (TR) ile Phone "541-123-45!" → "Invalid phone number." görüntülendi, kayıt yapılmadı.</t>
+          <t>Country Code +90 (TR), Phone "541-123-45!" → "Invalid phone number." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J638" s="8" t="n"/>
@@ -17420,7 +17420,7 @@
       </c>
       <c r="I660" s="4" t="inlineStr">
         <is>
-          <t>+90 (TR) ile Phone "54112345 (8 hane)" → "Invalid phone number." görüntülendi, kayıt yapılmadı.</t>
+          <t>Country Code +90 (TR), Phone "54112345 (8 hane)" → "Invalid phone number." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J660" s="8" t="n"/>
@@ -17972,7 +17972,7 @@
       </c>
       <c r="I682" s="4" t="inlineStr">
         <is>
-          <t>+90 (TR) ile Phone "541123456789 (12 hane)" → "Invalid phone number." görüntülendi, kayıt yapılmadı.</t>
+          <t>Country Code +90 (TR), Phone "541123456789 (12 hane)" → "Invalid phone number." görüntülendi, kayıt yapılmadı.</t>
         </is>
       </c>
       <c r="J682" s="8" t="n"/>
@@ -18524,7 +18524,7 @@
       </c>
       <c r="I704" s="4" t="inlineStr">
         <is>
-          <t>+1 (US) seçili, Phone "5411234567" (TR numarası) → "Invalid phone number." görüntülendi.</t>
+          <t>Country Code +1 (US) seçili, Phone "5411234567" (TR numarası) → "Invalid phone number." görüntülendi.</t>
         </is>
       </c>
       <c r="J704" s="8" t="n"/>

</xml_diff>